<commit_message>
Separate neocloud vs colocation; add Utilization & Rental Rates tab
- Split the 'leased' bucket into (a) leased COLOCATION (Meta leases
  space/power, owns the compute; in the electricity split) and (b)
  NEOCLOUD/CLOUD compute-as-a-service (provider owns the GPUs; $-based).
- New 'Neocloud & Cloud' tab: CoreWeave (~$35B), Nebius (up to $27B),
  Google Cloud ($10B+), AWS/Azure.
- New 'Utilization & Rental Rates' tab: colocation $/kW/mo by tier and
  metro + vacancy/occupancy (CBRE/JLL/CREFC); neocloud $/GPU-hr by SKU/
  provider + utilization economics (break-even, MFU, active vs contracted).
- Updated Summary (neocloud commitments block + taxonomy), Cover, and
  Sources; renamed 'Leased & Colocation' tab to 'Colocation (space & power)'.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/meta-compute-capacity/Meta_Compute_Capacity_Owned_vs_Leased.xlsx
+++ b/meta-compute-capacity/Meta_Compute_Capacity_Owned_vs_Leased.xlsx
@@ -11,9 +11,11 @@
     <sheet name="Summary - Owned vs Leased" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Owned - Site Energy" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Owned - Campus Detail" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Leased &amp; Colocation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="AI Buildout (GW)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sources &amp; Methodology" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Colocation (space &amp; power)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Neocloud &amp; Cloud" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Utilization &amp; Rental Rates" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="AI Buildout (GW)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Sources &amp; Methodology" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +24,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +76,13 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -113,7 +121,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EAF0FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF8F00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
       </patternFill>
     </fill>
   </fills>
@@ -187,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -232,12 +260,24 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -255,22 +295,43 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -278,9 +339,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -543,7 +601,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2700000"/>
@@ -565,7 +623,7 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="2700000"/>
@@ -875,7 +933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -922,56 +980,80 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Headline (FY2024, by electricity consumed)</t>
+          <t>Three procurement modes — the key distinction</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Owned online data centers: 14.89 TWh (~82%)  |  Leased/colocation: 3.07 TWh (~17%)  |  Other DC-related: 0.10 TWh (~1%).  Total data-center electricity = 18.06 TWh. Leased share has roughly doubled since 2020-22 (~9-11%) as Meta pre-leased heavily for AI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+          <t>Meta's compute is sourced three ways: (1) OWNED self-build data centers; (2) LEASED COLOCATION — Meta leases physical space &amp; power (powered shells / wholesale colo) from REITs/operators and installs its OWN servers/GPUs (measured in MW &amp; sqft; shows up in Meta's leased-facility electricity); and (3) NEOCLOUD / CLOUD — Meta rents GPU compute-as-a-service, where a THIRD PARTY owns the GPUs &amp; the building (measured in $ multi-year commitments / GPU-hours; it is opex, not in Meta's owned-electricity reporting). This workbook now separates colocation from neocloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Forward-looking AI capacity</t>
+          <t>Headline #1 — physical footprint (FY2024, by electricity consumed)</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Realized power today is dwarfed by the announced AI build-out. Trackers count ~15.8 GW of Meta AI data-center capacity across ~20 sites (~50% operational). Flagship clusters: Prometheus (Ohio, ~1 GW) and Hyperion (Louisiana, 2 GW scaling to 5 GW). Hyperion uses a $27-30B Blue Owl JV (Meta ~20% equity) that is leased back to Meta — an owned/leased hybrid. See 'AI Buildout' tab.</t>
+          <t>Owned online data centers: 14.89 TWh (~82%)  |  Leased colocation: 3.07 TWh (~17%)  |  Other DC-related: 0.10 TWh (~1%).  Total data-center electricity = 18.06 TWh. Leased colocation share roughly doubled since 2020-22 (~9-11%) as Meta pre-leased heavily for AI.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>Headline #2 — neocloud / cloud commitments ($, off the electricity split)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>CoreWeave ~$35B (initial $14.2B Sep-2025 + $21B expansion Apr-2026, through 2032; GB300 / Vera Rubin) | Nebius up to $27B ($12B fixed + $15B option) | Google Cloud $10B+ over 6 yrs (Aug-2025) | plus ongoing AWS &amp; Azure. ~$57B+ disclosed (up to ~$72B with options). These are compute rentals, NOT part of the owned-vs-colocation electricity split (different unit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Forward-looking AI capacity</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Realized power today is dwarfed by the announced AI build-out. Trackers count ~15.8 GW of Meta AI data-center capacity across ~20 sites (~50% operational). Flagship clusters: Prometheus (Ohio, ~1 GW) and Hyperion (Louisiana, 2 GW scaling to 5 GW). Hyperion uses a $27-30B Blue Owl JV (Meta ~20% equity) that is leased back to Meta — an owned/leased hybrid. See 'AI Buildout' tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>Tabs</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>1) Summary — owned vs leased split &amp; trend (authoritative, energy-based).  2) Owned - Site Energy — per-site MWh 2020-24.  3) Owned - Campus Detail — buildings, sqft, investment, nameplate MW est.  4) Leased &amp; Colocation — leased energy trend + markets.  5) AI Buildout (GW) — forward capacity.  6) Sources &amp; Methodology.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>1) Summary — owned vs colocation vs neocloud.  2) Owned - Site Energy — per-site MWh 2020-24.  3) Owned - Campus Detail — buildings, sqft, investment, nameplate MW est.  4) Colocation (space &amp; power) — leased-facility energy trend + markets.  5) Neocloud &amp; Cloud — GPU-as-a-service commitments.  6) Utilization &amp; Rental Rates — colocation ($/kW/mo, vacancy) &amp; neocloud ($/GPU-hr, utilization).  7) AI Buildout (GW).  8) Sources &amp; Methodology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Important caveats</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>• Electricity consumption ≠ nameplate MW, but is the best public realized-capacity proxy and is Meta-reported &amp; third-party assured.  • Nameplate MW figures (Campus Detail) are third-party estimates (usdatamap) and are incomplete — they predate/understate the AI expansion.  • GW figures for AI clusters are targets/announcements, not installed capacity.  • FY2024 = Jan 1 - Dec 31, 2024. All figures are as-disclosed and rounded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>• Electricity consumption ≠ nameplate MW, but is the best public realized-capacity proxy and is Meta-reported &amp; third-party assured.  • Colocation and neocloud are measured in DIFFERENT units (MWh vs $) and are not additive.  • Neocloud $ are multi-year contract values, not annual spend or installed capacity.  • Rental rates &amp; utilization on tab 6 are market benchmarks (CBRE/JLL/CREFC/neocloud disclosures), not Meta-specific contract terms, which are confidential.  • GW figures for AI clusters are targets/announcements.  • FY2024 = calendar 2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Units: MWh = megawatt-hours (energy/yr) · MW = megawatts (power) · GW = 1,000 MW · TWh = 1,000,000 MWh · sqft = square feet</t>
         </is>
@@ -992,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1115,7 +1197,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Leased data center facilities</t>
+          <t>Leased colocation facilities (Meta owns the compute)</t>
         </is>
       </c>
       <c r="B7" s="14" t="n">
@@ -1320,14 +1402,224 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Neocloud / third-party cloud commitments ($ multi-year) — separate from the electricity split above</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Counterparty</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Announced</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Value ($B)</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>CoreWeave — initial</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Neocloud (GPU-as-a-service)</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>Sep 2025</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>through Dec 14, 2031 (option to 2032)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>CoreWeave — expansion</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Neocloud (GPU-as-a-service)</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>2027-2032</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Neocloud (GPU-as-a-service)</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>multi-year (+$15B option)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Google Cloud</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>Aug 2025</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>6 years</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>Microsoft Azure</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Total disclosed neocloud/cloud commitments</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="n"/>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="31">
+        <f>SUMIF(D19:D24,"&lt;&gt;n/d")</f>
+        <v/>
+      </c>
+      <c r="E25" s="30" t="n"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Taxonomy: OWNED = Meta builds &amp; owns the DC and compute. COLOCATION = Meta leases space/power, owns the compute (in electricity split above, amber). NEOCLOUD/CLOUD = Meta rents GPU compute-as-a-service; the provider owns the GPUs &amp; building (this block, orange; measured in $, not MWh — not additive with the table above). See Neocloud &amp; Cloud and Utilization &amp; Rental Rates tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>Note: 'compute capacity' proxied by realized electricity consumption; see Cover &amp; Sources.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -1449,19 +1741,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="D5" s="32" t="n">
         <v>980000</v>
       </c>
-      <c r="E5" s="26" t="n">
+      <c r="E5" s="32" t="n">
         <v>950705</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="32" t="n">
         <v>1043606</v>
       </c>
-      <c r="G5" s="26" t="n">
+      <c r="G5" s="32" t="n">
         <v>1243306</v>
       </c>
-      <c r="H5" s="26" t="n">
+      <c r="H5" s="32" t="n">
         <v>1585392</v>
       </c>
       <c r="I5" s="25">
@@ -1470,37 +1762,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>Prineville</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>US-West</t>
         </is>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="34" t="n">
         <v>686000</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="34" t="n">
         <v>898409</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="34" t="n">
         <v>982177</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="34" t="n">
         <v>1375321</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="34" t="n">
         <v>1728291</v>
       </c>
-      <c r="I6" s="29">
+      <c r="I6" s="35">
         <f>H6/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1521,19 +1813,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="32" t="n">
         <v>519000</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="32" t="n">
         <v>736810</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="32" t="n">
         <v>1007635</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="32" t="n">
         <v>1148091</v>
       </c>
-      <c r="H7" s="26" t="n">
+      <c r="H7" s="32" t="n">
         <v>1258239</v>
       </c>
       <c r="I7" s="25">
@@ -1542,37 +1834,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Stanton Springs</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="34" t="n">
         <v>215279</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="34" t="n">
         <v>636266</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="34" t="n">
         <v>968565</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="34" t="n">
         <v>1184380</v>
       </c>
-      <c r="I8" s="29">
+      <c r="I8" s="35">
         <f>H8/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1593,19 +1885,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="D9" s="32" t="n">
         <v>571000</v>
       </c>
-      <c r="E9" s="26" t="n">
+      <c r="E9" s="32" t="n">
         <v>717932</v>
       </c>
-      <c r="F9" s="26" t="n">
+      <c r="F9" s="32" t="n">
         <v>929488</v>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="32" t="n">
         <v>1110100</v>
       </c>
-      <c r="H9" s="26" t="n">
+      <c r="H9" s="32" t="n">
         <v>1143067</v>
       </c>
       <c r="I9" s="25">
@@ -1614,37 +1906,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Eagle Mountain</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>US-West</t>
         </is>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="28" t="n">
+      <c r="E10" s="34" t="n">
         <v>229946</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="34" t="n">
         <v>504049</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="34" t="n">
         <v>787740</v>
       </c>
-      <c r="H10" s="28" t="n">
+      <c r="H10" s="34" t="n">
         <v>1115619</v>
       </c>
-      <c r="I10" s="29">
+      <c r="I10" s="35">
         <f>H10/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1665,19 +1957,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="32" t="n">
         <v>941000</v>
       </c>
-      <c r="E11" s="26" t="n">
+      <c r="E11" s="32" t="n">
         <v>1014447</v>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="32" t="n">
         <v>959419</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="32" t="n">
         <v>1029570</v>
       </c>
-      <c r="H11" s="26" t="n">
+      <c r="H11" s="32" t="n">
         <v>1109004</v>
       </c>
       <c r="I11" s="25">
@@ -1686,37 +1978,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Clonee</t>
         </is>
       </c>
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="34" t="n">
         <v>487000</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="34" t="n">
         <v>634648</v>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="34" t="n">
         <v>668290</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="34" t="n">
         <v>953837</v>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="34" t="n">
         <v>1076961</v>
       </c>
-      <c r="I12" s="29">
+      <c r="I12" s="35">
         <f>H12/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1737,19 +2029,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D13" s="26" t="n">
+      <c r="D13" s="32" t="n">
         <v>204000</v>
       </c>
-      <c r="E13" s="26" t="n">
+      <c r="E13" s="32" t="n">
         <v>515270</v>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="32" t="n">
         <v>701003</v>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="32" t="n">
         <v>805061</v>
       </c>
-      <c r="H13" s="26" t="n">
+      <c r="H13" s="32" t="n">
         <v>948859</v>
       </c>
       <c r="I13" s="25">
@@ -1758,37 +2050,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>Huntsville</t>
         </is>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D14" s="28" t="n">
+      <c r="D14" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="28" t="n">
+      <c r="E14" s="34" t="n">
         <v>85286</v>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="34" t="n">
         <v>368841</v>
       </c>
-      <c r="G14" s="28" t="n">
+      <c r="G14" s="34" t="n">
         <v>614198</v>
       </c>
-      <c r="H14" s="28" t="n">
+      <c r="H14" s="34" t="n">
         <v>865803</v>
       </c>
-      <c r="I14" s="29">
+      <c r="I14" s="35">
         <f>H14/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1809,19 +2101,19 @@
           <t>Denmark</t>
         </is>
       </c>
-      <c r="D15" s="26" t="n">
+      <c r="D15" s="32" t="n">
         <v>343000</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="32" t="n">
         <v>500863</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="32" t="n">
         <v>517718</v>
       </c>
-      <c r="G15" s="26" t="n">
+      <c r="G15" s="32" t="n">
         <v>518005</v>
       </c>
-      <c r="H15" s="26" t="n">
+      <c r="H15" s="32" t="n">
         <v>569374</v>
       </c>
       <c r="I15" s="25">
@@ -1830,37 +2122,37 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Forest City</t>
         </is>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D16" s="28" t="n">
+      <c r="D16" s="34" t="n">
         <v>595000</v>
       </c>
-      <c r="E16" s="28" t="n">
+      <c r="E16" s="34" t="n">
         <v>580842</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="34" t="n">
         <v>492786</v>
       </c>
-      <c r="G16" s="28" t="n">
+      <c r="G16" s="34" t="n">
         <v>507068</v>
       </c>
-      <c r="H16" s="28" t="n">
+      <c r="H16" s="34" t="n">
         <v>535555</v>
       </c>
-      <c r="I16" s="29">
+      <c r="I16" s="35">
         <f>H16/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1881,19 +2173,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D17" s="26" t="n">
+      <c r="D17" s="32" t="n">
         <v>270000</v>
       </c>
-      <c r="E17" s="26" t="n">
+      <c r="E17" s="32" t="n">
         <v>511414</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="32" t="n">
         <v>702694</v>
       </c>
-      <c r="G17" s="26" t="n">
+      <c r="G17" s="32" t="n">
         <v>793063</v>
       </c>
-      <c r="H17" s="26" t="n">
+      <c r="H17" s="32" t="n">
         <v>521217</v>
       </c>
       <c r="I17" s="25">
@@ -1902,37 +2194,37 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>Luleå</t>
         </is>
       </c>
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>Sweden</t>
         </is>
       </c>
-      <c r="D18" s="28" t="n">
+      <c r="D18" s="34" t="n">
         <v>369000</v>
       </c>
-      <c r="E18" s="28" t="n">
+      <c r="E18" s="34" t="n">
         <v>306054</v>
       </c>
-      <c r="F18" s="28" t="n">
+      <c r="F18" s="34" t="n">
         <v>267471</v>
       </c>
-      <c r="G18" s="28" t="n">
+      <c r="G18" s="34" t="n">
         <v>351931</v>
       </c>
-      <c r="H18" s="28" t="n">
+      <c r="H18" s="34" t="n">
         <v>468809</v>
       </c>
-      <c r="I18" s="29">
+      <c r="I18" s="35">
         <f>H18/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -1953,19 +2245,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D19" s="26" t="n">
+      <c r="D19" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="26" t="n">
+      <c r="E19" s="32" t="n">
         <v>4724</v>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F19" s="32" t="n">
         <v>16934</v>
       </c>
-      <c r="G19" s="26" t="n">
+      <c r="G19" s="32" t="n">
         <v>138965</v>
       </c>
-      <c r="H19" s="26" t="n">
+      <c r="H19" s="32" t="n">
         <v>372339</v>
       </c>
       <c r="I19" s="25">
@@ -1974,37 +2266,37 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>Gallatin</t>
         </is>
       </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D20" s="28" t="n">
+      <c r="D20" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="28" t="n">
+      <c r="E20" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="28" t="n">
+      <c r="F20" s="34" t="n">
         <v>6264</v>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="G20" s="34" t="n">
         <v>116520</v>
       </c>
-      <c r="H20" s="28" t="n">
+      <c r="H20" s="34" t="n">
         <v>359730</v>
       </c>
-      <c r="I20" s="29">
+      <c r="I20" s="35">
         <f>H20/SUM($H$5:$H$22)</f>
         <v/>
       </c>
@@ -2025,19 +2317,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D21" s="26" t="n">
+      <c r="D21" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="26" t="n">
+      <c r="E21" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F21" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="26" t="n">
+      <c r="G21" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="26" t="n">
+      <c r="H21" s="32" t="n">
         <v>24657</v>
       </c>
       <c r="I21" s="25">
@@ -2046,117 +2338,117 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Kansas City</t>
         </is>
       </c>
-      <c r="B22" s="27" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>US-Midwest</t>
         </is>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D22" s="28" t="n">
+      <c r="D22" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="28" t="n">
+      <c r="E22" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="28" t="n">
+      <c r="F22" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="28" t="n">
+      <c r="G22" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="28" t="n">
+      <c r="H22" s="34" t="n">
         <v>22963</v>
       </c>
-      <c r="I22" s="29">
+      <c r="I22" s="35">
         <f>H22/SUM($H$5:$H$22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Total owned online data centers</t>
         </is>
       </c>
-      <c r="B23" s="30" t="inlineStr"/>
-      <c r="C23" s="30" t="n"/>
-      <c r="D23" s="31">
+      <c r="B23" s="36" t="inlineStr"/>
+      <c r="C23" s="36" t="n"/>
+      <c r="D23" s="37">
         <f>SUM(D5:D22)</f>
         <v/>
       </c>
-      <c r="E23" s="31">
+      <c r="E23" s="37">
         <f>SUM(E5:E22)</f>
         <v/>
       </c>
-      <c r="F23" s="31">
+      <c r="F23" s="37">
         <f>SUM(F5:F22)</f>
         <v/>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="37">
         <f>SUM(G5:G22)</f>
         <v/>
       </c>
-      <c r="H23" s="31">
+      <c r="H23" s="37">
         <f>SUM(H5:H22)</f>
         <v/>
       </c>
-      <c r="I23" s="32">
+      <c r="I23" s="38">
         <f>SUM(I5:I22)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="33" t="inlineStr">
-        <is>
-          <t>Memo — Leased data center facilities</t>
-        </is>
-      </c>
-      <c r="B25" s="34" t="n"/>
-      <c r="C25" s="34" t="n"/>
-      <c r="D25" s="35" t="n">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>Memo — Leased colocation facilities</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n"/>
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="41" t="n">
         <v>795000</v>
       </c>
-      <c r="E25" s="35" t="n">
+      <c r="E25" s="41" t="n">
         <v>964650</v>
       </c>
-      <c r="F25" s="35" t="n">
+      <c r="F25" s="41" t="n">
         <v>1105834</v>
       </c>
-      <c r="G25" s="35" t="n">
+      <c r="G25" s="41" t="n">
         <v>2187020</v>
       </c>
-      <c r="H25" s="35" t="n">
+      <c r="H25" s="41" t="n">
         <v>3069504</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="36" t="inlineStr">
+      <c r="A26" s="42" t="inlineStr">
         <is>
           <t>Memo — Other DC-related facilities</t>
         </is>
       </c>
-      <c r="D26" s="37" t="n">
+      <c r="D26" s="43" t="n">
         <v>206000</v>
       </c>
-      <c r="E26" s="37" t="n">
+      <c r="E26" s="43" t="n">
         <v>249843</v>
       </c>
-      <c r="F26" s="37" t="n">
+      <c r="F26" s="43" t="n">
         <v>256939</v>
       </c>
-      <c r="G26" s="37" t="n">
+      <c r="G26" s="43" t="n">
         <v>327073</v>
       </c>
-      <c r="H26" s="37" t="n">
+      <c r="H26" s="43" t="n">
         <v>102016</v>
       </c>
     </row>
@@ -2282,19 +2574,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="44" t="n">
         <v>2011</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="E5" s="45" t="n">
         <v>11</v>
       </c>
-      <c r="F5" s="40" t="n">
+      <c r="F5" s="46" t="n">
         <v>4.6</v>
       </c>
-      <c r="G5" s="40" t="n">
+      <c r="G5" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="39" t="n">
+      <c r="H5" s="45" t="n">
         <v>180</v>
       </c>
       <c r="I5" s="24" t="inlineStr">
@@ -2304,37 +2596,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>Forest City, NC</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D6" s="41" t="n">
+      <c r="D6" s="47" t="n">
         <v>2012</v>
       </c>
-      <c r="E6" s="42" t="n">
+      <c r="E6" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="49" t="n">
         <v>1.3</v>
       </c>
-      <c r="G6" s="43" t="n">
+      <c r="G6" s="49" t="n">
         <v>0.8</v>
       </c>
-      <c r="H6" s="42" t="n">
+      <c r="H6" s="48" t="n">
         <v>160</v>
       </c>
-      <c r="I6" s="27" t="inlineStr">
+      <c r="I6" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2356,19 +2648,19 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="44" t="n">
         <v>2013</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="E7" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="40" t="n">
+      <c r="F7" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="40" t="n">
+      <c r="G7" s="46" t="n">
         <v>0.8</v>
       </c>
-      <c r="H7" s="38" t="inlineStr">
+      <c r="H7" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -2380,37 +2672,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Altoona, IA</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>US-Midwest</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D8" s="41" t="n">
+      <c r="D8" s="47" t="n">
         <v>2014</v>
       </c>
-      <c r="E8" s="42" t="n">
+      <c r="E8" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="49" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="43" t="n">
+      <c r="G8" s="49" t="n">
         <v>2.5</v>
       </c>
-      <c r="H8" s="42" t="n">
+      <c r="H8" s="48" t="n">
         <v>200</v>
       </c>
-      <c r="I8" s="27" t="inlineStr">
+      <c r="I8" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2432,19 +2724,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="44" t="n">
         <v>2017</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="E9" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="40" t="n">
+      <c r="F9" s="46" t="n">
         <v>2.6</v>
       </c>
-      <c r="G9" s="40" t="n">
+      <c r="G9" s="46" t="n">
         <v>1.5</v>
       </c>
-      <c r="H9" s="38" t="inlineStr">
+      <c r="H9" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -2456,39 +2748,39 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Clonee, Ireland</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="47" t="n">
         <v>2018</v>
       </c>
-      <c r="E10" s="42" t="n">
+      <c r="E10" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="43" t="n">
+      <c r="F10" s="49" t="n">
         <v>1.6</v>
       </c>
-      <c r="G10" s="43" t="n">
+      <c r="G10" s="49" t="n">
         <v>1.5</v>
       </c>
-      <c r="H10" s="41" t="inlineStr">
+      <c r="H10" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I10" s="27" t="inlineStr">
+      <c r="I10" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2510,19 +2802,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="44" t="n">
         <v>2019</v>
       </c>
-      <c r="E11" s="39" t="n">
+      <c r="E11" s="45" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="40" t="n">
+      <c r="F11" s="46" t="n">
         <v>3.8</v>
       </c>
-      <c r="G11" s="40" t="n">
+      <c r="G11" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="39" t="n">
+      <c r="H11" s="45" t="n">
         <v>100</v>
       </c>
       <c r="I11" s="24" t="inlineStr">
@@ -2532,39 +2824,39 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Odense, Denmark</t>
         </is>
       </c>
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>Denmark</t>
         </is>
       </c>
-      <c r="D12" s="41" t="n">
+      <c r="D12" s="47" t="n">
         <v>2019</v>
       </c>
-      <c r="E12" s="42" t="n">
+      <c r="E12" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="43" t="n">
+      <c r="F12" s="49" t="n">
         <v>0.9</v>
       </c>
-      <c r="G12" s="43" t="n">
+      <c r="G12" s="49" t="n">
         <v>1.9</v>
       </c>
-      <c r="H12" s="41" t="inlineStr">
+      <c r="H12" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I12" s="27" t="inlineStr">
+      <c r="I12" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2586,19 +2878,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D13" s="38" t="n">
+      <c r="D13" s="44" t="n">
         <v>2019</v>
       </c>
-      <c r="E13" s="39" t="n">
+      <c r="E13" s="45" t="n">
         <v>9</v>
       </c>
-      <c r="F13" s="40" t="n">
+      <c r="F13" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="40" t="n">
+      <c r="G13" s="46" t="n">
         <v>1.5</v>
       </c>
-      <c r="H13" s="39" t="n">
+      <c r="H13" s="45" t="n">
         <v>80</v>
       </c>
       <c r="I13" s="24" t="inlineStr">
@@ -2608,37 +2900,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>New Albany, OH</t>
         </is>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>US-Midwest</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D14" s="41" t="n">
+      <c r="D14" s="47" t="n">
         <v>2020</v>
       </c>
-      <c r="E14" s="42" t="n">
+      <c r="E14" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="43" t="n">
+      <c r="F14" s="49" t="n">
         <v>2.5</v>
       </c>
-      <c r="G14" s="43" t="n">
+      <c r="G14" s="49" t="n">
         <v>1.5</v>
       </c>
-      <c r="H14" s="42" t="n">
+      <c r="H14" s="48" t="n">
         <v>250</v>
       </c>
-      <c r="I14" s="27" t="inlineStr">
+      <c r="I14" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2660,19 +2952,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D15" s="38" t="n">
+      <c r="D15" s="44" t="n">
         <v>2020</v>
       </c>
-      <c r="E15" s="39" t="n">
+      <c r="E15" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="40" t="n">
+      <c r="F15" s="46" t="n">
         <v>2.5</v>
       </c>
-      <c r="G15" s="40" t="n">
+      <c r="G15" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="39" t="n">
+      <c r="H15" s="45" t="n">
         <v>200</v>
       </c>
       <c r="I15" s="24" t="inlineStr">
@@ -2682,37 +2974,37 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D16" s="41" t="n">
+      <c r="D16" s="47" t="n">
         <v>2021</v>
       </c>
-      <c r="E16" s="42" t="n">
+      <c r="E16" s="48" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="43" t="n">
+      <c r="F16" s="49" t="n">
         <v>3.5</v>
       </c>
-      <c r="G16" s="43" t="n">
+      <c r="G16" s="49" t="n">
         <v>1.5</v>
       </c>
-      <c r="H16" s="42" t="n">
+      <c r="H16" s="48" t="n">
         <v>120</v>
       </c>
-      <c r="I16" s="27" t="inlineStr">
+      <c r="I16" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2734,19 +3026,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D17" s="38" t="n">
+      <c r="D17" s="44" t="n">
         <v>2021</v>
       </c>
-      <c r="E17" s="39" t="n">
+      <c r="E17" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F17" s="40" t="n">
+      <c r="F17" s="46" t="n">
         <v>2.5</v>
       </c>
-      <c r="G17" s="40" t="n">
+      <c r="G17" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="39" t="n">
+      <c r="H17" s="45" t="n">
         <v>200</v>
       </c>
       <c r="I17" s="24" t="inlineStr">
@@ -2756,39 +3048,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>Eagle Mountain, UT</t>
         </is>
       </c>
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>US-West</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D18" s="41" t="n">
+      <c r="D18" s="47" t="n">
         <v>2021</v>
       </c>
-      <c r="E18" s="42" t="n">
+      <c r="E18" s="48" t="n">
         <v>7</v>
       </c>
-      <c r="F18" s="43" t="n">
+      <c r="F18" s="49" t="n">
         <v>4.5</v>
       </c>
-      <c r="G18" s="43" t="n">
+      <c r="G18" s="49" t="n">
         <v>1.5</v>
       </c>
-      <c r="H18" s="41" t="inlineStr">
+      <c r="H18" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I18" s="27" t="inlineStr">
+      <c r="I18" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2810,19 +3102,19 @@
           <t>Singapore</t>
         </is>
       </c>
-      <c r="D19" s="38" t="n">
+      <c r="D19" s="44" t="n">
         <v>2022</v>
       </c>
-      <c r="E19" s="39" t="n">
+      <c r="E19" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="40" t="n">
+      <c r="F19" s="46" t="n">
         <v>1.8</v>
       </c>
-      <c r="G19" s="40" t="n">
+      <c r="G19" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="38" t="inlineStr">
+      <c r="H19" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -2834,37 +3126,37 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>DeKalb, IL</t>
         </is>
       </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="33" t="inlineStr">
         <is>
           <t>US-Midwest</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="47" t="n">
         <v>2022</v>
       </c>
-      <c r="E20" s="42" t="n">
+      <c r="E20" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="F20" s="43" t="n">
+      <c r="F20" s="49" t="n">
         <v>2.4</v>
       </c>
-      <c r="G20" s="43" t="n">
+      <c r="G20" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="42" t="n">
+      <c r="H20" s="48" t="n">
         <v>300</v>
       </c>
-      <c r="I20" s="27" t="inlineStr">
+      <c r="I20" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2886,19 +3178,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D21" s="38" t="n">
+      <c r="D21" s="44" t="n">
         <v>2023</v>
       </c>
-      <c r="E21" s="39" t="n">
+      <c r="E21" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="40" t="n">
+      <c r="F21" s="46" t="n">
         <v>1.6</v>
       </c>
-      <c r="G21" s="40" t="n">
+      <c r="G21" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="38" t="inlineStr">
+      <c r="H21" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -2910,39 +3202,39 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Mesa, AZ</t>
         </is>
       </c>
-      <c r="B22" s="27" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>US-Southwest</t>
         </is>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D22" s="47" t="n">
         <v>2023</v>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E22" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="F22" s="43" t="n">
+      <c r="F22" s="49" t="n">
         <v>2.5</v>
       </c>
-      <c r="G22" s="43" t="n">
+      <c r="G22" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="41" t="inlineStr">
+      <c r="H22" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I22" s="27" t="inlineStr">
+      <c r="I22" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -2964,19 +3256,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D23" s="38" t="n">
+      <c r="D23" s="44" t="n">
         <v>2024</v>
       </c>
-      <c r="E23" s="39" t="n">
+      <c r="E23" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="40" t="n">
+      <c r="F23" s="46" t="n">
         <v>0.9</v>
       </c>
-      <c r="G23" s="40" t="n">
+      <c r="G23" s="46" t="n">
         <v>0.8</v>
       </c>
-      <c r="H23" s="38" t="inlineStr">
+      <c r="H23" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -2988,39 +3280,39 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>Kansas City, MO</t>
         </is>
       </c>
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B24" s="33" t="inlineStr">
         <is>
           <t>US-Midwest</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C24" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="47" t="n">
         <v>2024</v>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E24" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="43" t="n">
+      <c r="F24" s="49" t="n">
         <v>0.7</v>
       </c>
-      <c r="G24" s="43" t="n">
+      <c r="G24" s="49" t="n">
         <v>0.8</v>
       </c>
-      <c r="H24" s="41" t="inlineStr">
+      <c r="H24" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I24" s="27" t="inlineStr">
+      <c r="I24" s="33" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
@@ -3042,19 +3334,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D25" s="38" t="n">
+      <c r="D25" s="44" t="n">
         <v>2025</v>
       </c>
-      <c r="E25" s="39" t="n">
+      <c r="E25" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="40" t="n">
+      <c r="F25" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="40" t="n">
+      <c r="G25" s="46" t="n">
         <v>0.8</v>
       </c>
-      <c r="H25" s="39" t="n">
+      <c r="H25" s="45" t="n">
         <v>100</v>
       </c>
       <c r="I25" s="24" t="inlineStr">
@@ -3064,39 +3356,39 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t>Jeffersonville, IN</t>
         </is>
       </c>
-      <c r="B26" s="27" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>US-Midwest</t>
         </is>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="47" t="n">
         <v>2026</v>
       </c>
-      <c r="E26" s="42" t="n">
+      <c r="E26" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="43" t="n">
+      <c r="F26" s="49" t="n">
         <v>0.7</v>
       </c>
-      <c r="G26" s="43" t="n">
+      <c r="G26" s="49" t="n">
         <v>0.8</v>
       </c>
-      <c r="H26" s="41" t="inlineStr">
+      <c r="H26" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I26" s="27" t="inlineStr">
+      <c r="I26" s="33" t="inlineStr">
         <is>
           <t>Under construction</t>
         </is>
@@ -3118,19 +3410,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="D27" s="38" t="n">
+      <c r="D27" s="44" t="n">
         <v>2026</v>
       </c>
-      <c r="E27" s="39" t="n">
+      <c r="E27" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="40" t="n">
+      <c r="F27" s="46" t="n">
         <v>0.72</v>
       </c>
-      <c r="G27" s="40" t="n">
+      <c r="G27" s="46" t="n">
         <v>0.8</v>
       </c>
-      <c r="H27" s="38" t="inlineStr">
+      <c r="H27" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -3142,70 +3434,70 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>Montgomery, AL</t>
         </is>
       </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B28" s="33" t="inlineStr">
         <is>
           <t>US-Southeast</t>
         </is>
       </c>
-      <c r="C28" s="27" t="inlineStr">
+      <c r="C28" s="33" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="47" t="n">
         <v>2026</v>
       </c>
-      <c r="E28" s="42" t="n">
+      <c r="E28" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F28" s="43" t="n">
+      <c r="F28" s="49" t="n">
         <v>0.72</v>
       </c>
-      <c r="G28" s="43" t="n">
+      <c r="G28" s="49" t="n">
         <v>0.8</v>
       </c>
-      <c r="H28" s="41" t="inlineStr">
+      <c r="H28" s="47" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I28" s="27" t="inlineStr">
+      <c r="I28" s="33" t="inlineStr">
         <is>
           <t>Under construction</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="30" t="inlineStr">
+      <c r="A29" s="36" t="inlineStr">
         <is>
           <t>TOTAL (owned campuses)</t>
         </is>
       </c>
-      <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="31">
+      <c r="B29" s="36" t="n"/>
+      <c r="C29" s="36" t="n"/>
+      <c r="D29" s="36" t="n"/>
+      <c r="E29" s="37">
         <f>SUM(E5:E28)</f>
         <v/>
       </c>
-      <c r="F29" s="44">
+      <c r="F29" s="50">
         <f>SUM(F5:F28)</f>
         <v/>
       </c>
-      <c r="G29" s="44">
+      <c r="G29" s="50">
         <f>SUM(G5:G28)</f>
         <v/>
       </c>
-      <c r="H29" s="31">
+      <c r="H29" s="37">
         <f>SUMIF(H5:H28,"&lt;&gt;n/a")</f>
         <v/>
       </c>
-      <c r="I29" s="30" t="n"/>
+      <c r="I29" s="36" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -3229,21 +3521,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Leased / Colocation Capacity</t>
+          <t>Leased Colocation — Space &amp; Power (Meta owns the compute)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -3255,7 +3547,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Third-party leased data-center facilities. Sources: Meta Environmental Data Index; Dgtl Infra; SemiAnalysis.</t>
+          <t>Meta leases powered shells / wholesale colo and installs its own servers. Sources: Meta Env. Data Index; Dgtl Infra; SemiAnalysis.</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -3264,295 +3556,1635 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Leased data-center electricity consumption (MWh/yr)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Definition: colocation = Meta rents physical data-center space &amp; power from third parties (REITs/operators) but owns and operates the servers/GPUs inside. It IS captured in Meta's 'Leased data center facilities' electricity line. (Contrast with neocloud — see next tab.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Leased colocation electricity consumption (MWh/yr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Leased facilities (MWh)</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Leased colocation facilities (MWh)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
         <v>795000</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C8" s="14" t="n">
         <v>964650</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D8" s="14" t="n">
         <v>1105834</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E8" s="14" t="n">
         <v>2187020</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F8" s="14" t="n">
         <v>3069504</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>YoY growth</t>
         </is>
       </c>
-      <c r="B7" s="38" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="C7" s="25">
-        <f>C6/B6-1</f>
+      <c r="C9" s="25">
+        <f>C8/B8-1</f>
         <v/>
       </c>
-      <c r="D7" s="25">
-        <f>D6/C6-1</f>
+      <c r="D9" s="25">
+        <f>D8/C8-1</f>
         <v/>
       </c>
-      <c r="E7" s="25">
-        <f>E6/D6-1</f>
+      <c r="E9" s="25">
+        <f>E8/D8-1</f>
         <v/>
       </c>
-      <c r="F7" s="25">
-        <f>F6/E6-1</f>
+      <c r="F9" s="25">
+        <f>F8/E8-1</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Known leased / colocation markets</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Known colocation markets (Meta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="C10" s="45" t="n"/>
-      <c r="D10" s="46" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="38" t="n">
+    </row>
+    <row r="13">
+      <c r="A13" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Ashburn, Virginia</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="38" t="n">
+    <row r="14">
+      <c r="A14" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Manassas, Virginia</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="38" t="n">
+    <row r="15">
+      <c r="A15" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>Richmond, Virginia</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="38" t="n">
+    <row r="16">
+      <c r="A16" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>Aurora, Illinois</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="38" t="n">
+    <row r="17">
+      <c r="A17" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Chicago, Illinois</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="38" t="n">
+    <row r="18">
+      <c r="A18" s="44" t="n">
         <v>6</v>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Dallas, Texas</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="38" t="n">
+    <row r="19">
+      <c r="A19" s="44" t="n">
         <v>7</v>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Houston, Texas</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="38" t="n">
+    <row r="20">
+      <c r="A20" s="44" t="n">
         <v>8</v>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Phoenix, Arizona</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="38" t="n">
+    <row r="21">
+      <c r="A21" s="44" t="n">
         <v>9</v>
       </c>
-      <c r="B19" s="24" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Hillsboro, Oregon</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="38" t="n">
+    <row r="22">
+      <c r="A22" s="44" t="n">
         <v>10</v>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Santa Clara, California</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="38" t="n">
+    <row r="23">
+      <c r="A23" s="44" t="n">
         <v>11</v>
       </c>
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Chennai, India</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Key relationships &amp; context</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>• Digital Realty (DLR): Meta is its ~11th-largest customer; ~48 leased locations; ~$61.8M annualized base rent (Dgtl Infra).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>• SemiAnalysis: Meta pre-leased more capacity in H2-2024 than any other hyperscaler, concentrated in Ohio.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>• Dual-track 'all of the above' strategy: self-build + leasing + on-site gas generation to ramp AI capacity fast.</t>
+          <t>• Digital Realty (DLR): Meta is its ~11th-largest customer; ~48 leased locations; ~$61.8M annualized base rent (Dgtl Infra).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>• Hyperion (Louisiana) is financed via a $27-30B Blue Owl JV (Meta ~20% equity) and leased back to Meta — an owned/leased hybrid (see AI Buildout).</t>
+          <t>• SemiAnalysis: Meta pre-leased more colocation capacity in H2-2024 than any other hyperscaler, concentrated in Ohio.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>• Leased DC electricity nearly quadrupled 2020-&gt;2024 (0.80 -&gt; 3.07 TWh); leased share of DC power rose from ~11% to ~17%.</t>
+          <t>• Dual-track 'all of the above' strategy: self-build + colocation leasing + neocloud + on-site gas generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>• Hyperion (Louisiana) is financed via a $27-30B Blue Owl JV (Meta ~20% equity) and leased back to Meta — an owned/leased hybrid (see AI Buildout).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>• Leased colocation electricity nearly quadrupled 2020-&gt;2024 (0.80 -&gt; 3.07 TWh); colocation share of DC power rose from ~11% to ~17%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>• Market rental rates &amp; utilization/vacancy for colocation are on the 'Utilization &amp; Rental Rates' tab.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B11:D11"/>
+  <mergeCells count="21">
     <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="A26:F26"/>
-    <mergeCell ref="B10:D10"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A4:F4"/>
     <mergeCell ref="B15:D15"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="B16:D16"/>
-    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B12:D12"/>
-    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Neocloud / Third-Party Cloud — Compute-as-a-Service</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Meta rents GPU capacity; the provider owns the GPUs &amp; building. Measured in $ commitments (opex), not Meta MWh.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Definition: neocloud/cloud = Meta buys managed GPU compute from a third party that owns the chips and data centers (CoreWeave, Nebius, Google Cloud, AWS, Azure). This is NOT in Meta's owned/colocation electricity split; it is a separate, $-denominated procurement channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Counterparty</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Announced</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Value ($B)</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Scope / hardware</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="51" t="inlineStr">
+        <is>
+          <t>CoreWeave — initial</t>
+        </is>
+      </c>
+      <c r="B7" s="51" t="inlineStr">
+        <is>
+          <t>Neocloud (GPU-as-a-service)</t>
+        </is>
+      </c>
+      <c r="C7" s="52" t="inlineStr">
+        <is>
+          <t>Sep 2025</t>
+        </is>
+      </c>
+      <c r="D7" s="53" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E7" s="51" t="inlineStr">
+        <is>
+          <t>through Dec 14, 2031 (option to 2032)</t>
+        </is>
+      </c>
+      <c r="F7" s="51" t="inlineStr">
+        <is>
+          <t>NVIDIA GB300 systems</t>
+        </is>
+      </c>
+      <c r="G7" s="51" t="inlineStr">
+        <is>
+          <t>First major Meta neocloud contract; disclosed in CoreWeave SEC filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="51" t="inlineStr">
+        <is>
+          <t>CoreWeave — expansion</t>
+        </is>
+      </c>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>Neocloud (GPU-as-a-service)</t>
+        </is>
+      </c>
+      <c r="C8" s="52" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t>2027-2032</t>
+        </is>
+      </c>
+      <c r="F8" s="51" t="inlineStr">
+        <is>
+          <t>Dedicated capacity, multi-site; incl. NVIDIA Vera Rubin</t>
+        </is>
+      </c>
+      <c r="G8" s="51" t="inlineStr">
+        <is>
+          <t>Brings Meta-CoreWeave total to ~$35B; supports large-scale AI inference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="51" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B9" s="51" t="inlineStr">
+        <is>
+          <t>Neocloud (GPU-as-a-service)</t>
+        </is>
+      </c>
+      <c r="C9" s="52" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D9" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" s="51" t="inlineStr">
+        <is>
+          <t>multi-year (+$15B option)</t>
+        </is>
+      </c>
+      <c r="F9" s="51" t="inlineStr">
+        <is>
+          <t>Fixed dedicated compute</t>
+        </is>
+      </c>
+      <c r="G9" s="51" t="inlineStr">
+        <is>
+          <t>Up to $27B including a $15B option exercisable at Nebius's discretion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="51" t="inlineStr">
+        <is>
+          <t>Google Cloud</t>
+        </is>
+      </c>
+      <c r="B10" s="51" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C10" s="52" t="inlineStr">
+        <is>
+          <t>Aug 2025</t>
+        </is>
+      </c>
+      <c r="D10" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="51" t="inlineStr">
+        <is>
+          <t>6 years</t>
+        </is>
+      </c>
+      <c r="F10" s="51" t="inlineStr">
+        <is>
+          <t>Servers, storage, networking for AI</t>
+        </is>
+      </c>
+      <c r="G10" s="51" t="inlineStr">
+        <is>
+          <t>Minimum ~$10B; mainly AI infrastructure scaling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="51" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="B11" s="51" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C11" s="52" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D11" s="52" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E11" s="51" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="F11" s="51" t="inlineStr">
+        <is>
+          <t>Cloud infrastructure</t>
+        </is>
+      </c>
+      <c r="G11" s="51" t="inlineStr">
+        <is>
+          <t>Long-standing; value undisclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="51" t="inlineStr">
+        <is>
+          <t>Microsoft Azure</t>
+        </is>
+      </c>
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C12" s="52" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D12" s="52" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="F12" s="51" t="inlineStr">
+        <is>
+          <t>Cloud infrastructure</t>
+        </is>
+      </c>
+      <c r="G12" s="51" t="inlineStr">
+        <is>
+          <t>Long-standing; value undisclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Total disclosed commitments</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="n"/>
+      <c r="C13" s="30" t="n"/>
+      <c r="D13" s="31">
+        <f>SUMIF(D7:D12,"&lt;&gt;n/d")</f>
+        <v/>
+      </c>
+      <c r="E13" s="30" t="n"/>
+      <c r="F13" s="30" t="n"/>
+      <c r="G13" s="30" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>• Meta describes this as a 'portfolio-based approach to infrastructure' — self-build + colocation + neocloud together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>• CoreWeave total with Meta ~$35B (through 2032); CoreWeave overall backlog $99.4B (Mar-2026) on &gt;3.5 GW contracted power.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>• Nebius Meta deal up to $27B: $12B fixed dedicated compute + $15B option (exercisable by Nebius).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>• Google Cloud: $10B+ / 6 yrs; Meta historically also uses AWS and Azure (values undisclosed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>• Neocloud GPU rental rates and utilization economics are on the 'Utilization &amp; Rental Rates' tab.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Utilization &amp; Rental Rates — Colocation vs Neocloud</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Market benchmarks (NOT Meta-specific contract terms, which are confidential). Sources: CBRE, JLL, CREFC, neocloud disclosures.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>A.  COLOCATION (space &amp; power leasing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Rental rates by deal tier ($/kW/month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Typical size</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Typical term</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Rate ($/kW/mo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Retail / edge colocation</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>&lt; ~250 kW</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>1-3 yr</t>
+        </is>
+      </c>
+      <c r="D7" s="55" t="inlineStr">
+        <is>
+          <t>$200 - $400</t>
+        </is>
+      </c>
+      <c r="E7" s="56" t="inlineStr">
+        <is>
+          <t>Highest unit price; smallest deployments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Wholesale colocation</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>~250 kW - a few MW</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>5-10 yr</t>
+        </is>
+      </c>
+      <c r="D8" s="55" t="inlineStr">
+        <is>
+          <t>$150 - $250</t>
+        </is>
+      </c>
+      <c r="E8" s="56" t="inlineStr">
+        <is>
+          <t>Mid-size; typical enterprise / AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Hyperscale / build-to-suit</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>5 - 40+ MW</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>10-15 yr</t>
+        </is>
+      </c>
+      <c r="D9" s="55" t="inlineStr">
+        <is>
+          <t>$100 - $150</t>
+        </is>
+      </c>
+      <c r="E9" s="56" t="inlineStr">
+        <is>
+          <t>Largest deals, lowest unit rate — Meta's tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Rental rates by market (250-500 kW requirement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Asking rate</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>YoY</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E12" s="57" t="n"/>
+      <c r="F12" s="58" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Primary N. America avg (250-500 kW)</t>
+        </is>
+      </c>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>~$196 / kW/mo</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="inlineStr">
+        <is>
+          <t>+6.6% YoY</t>
+        </is>
+      </c>
+      <c r="D13" s="59" t="inlineStr">
+        <is>
+          <t>CBRE H2-2025 record; 4th straight annual rise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>$200 - $230</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>+14.7% YoY</t>
+        </is>
+      </c>
+      <c r="D14" s="59" t="inlineStr">
+        <is>
+          <t>Highest US primary rate (Q1-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Northern Virginia</t>
+        </is>
+      </c>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t>$190 - $235</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>single-digit</t>
+        </is>
+      </c>
+      <c r="D15" s="59" t="inlineStr">
+        <is>
+          <t>Largest US market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>$160 - $180</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>+2% YoY</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>Fast-growing; vacancy ~1%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Dallas-Ft. Worth</t>
+        </is>
+      </c>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>market rate</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>~flat</t>
+        </is>
+      </c>
+      <c r="D17" s="59" t="inlineStr">
+        <is>
+          <t>Asking rents roughly unchanged YoY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>$235 - $265</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>up YoY</t>
+        </is>
+      </c>
+      <c r="D18" s="59" t="inlineStr">
+        <is>
+          <t>Highest European rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>$310 - $475</t>
+        </is>
+      </c>
+      <c r="C19" s="44" t="inlineStr">
+        <is>
+          <t>up YoY</t>
+        </is>
+      </c>
+      <c r="D19" s="59" t="inlineStr">
+        <is>
+          <t>Highest APAC rate; supply-constrained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>10 MW+ deployments</t>
+        </is>
+      </c>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>premium/scarce</t>
+        </is>
+      </c>
+      <c r="C20" s="44" t="inlineStr">
+        <is>
+          <t>up to +19% YoY</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr">
+        <is>
+          <t>Large contiguous blocks command premiums.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Utilization / occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="D23" s="57" t="n"/>
+      <c r="E23" s="57" t="n"/>
+      <c r="F23" s="58" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Primary-market vacancy (CBRE, YE2025)</t>
+        </is>
+      </c>
+      <c r="B24" s="55" t="inlineStr">
+        <is>
+          <t>1.4%</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="inlineStr">
+        <is>
+          <t>Record low.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Primary-market vacancy (JLL, YE2025)</t>
+        </is>
+      </c>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+      <c r="C25" s="59" t="inlineStr">
+        <is>
+          <t>2nd straight year; ~99% occupancy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Under-construction precommitted (JLL)</t>
+        </is>
+      </c>
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="C26" s="59" t="inlineStr">
+        <is>
+          <t>Binding leases or owner-occupied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Under-construction that is leased (JLL)</t>
+        </is>
+      </c>
+      <c r="B27" s="55" t="inlineStr">
+        <is>
+          <t>~60%</t>
+        </is>
+      </c>
+      <c r="C27" s="59" t="inlineStr">
+        <is>
+          <t>Remaining ~40% owner-occupied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>N. America capacity under construction (JLL)</t>
+        </is>
+      </c>
+      <c r="B28" s="55" t="inlineStr">
+        <is>
+          <t>35+ GW</t>
+        </is>
+      </c>
+      <c r="C28" s="59" t="inlineStr">
+        <is>
+          <t>Extraordinary by historical standards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Net absorption, primary markets 2025 (CBRE)</t>
+        </is>
+      </c>
+      <c r="B29" s="55" t="inlineStr">
+        <is>
+          <t>2,498 MW</t>
+        </is>
+      </c>
+      <c r="C29" s="59" t="inlineStr">
+        <is>
+          <t>Record; prior peak 1,810 MW (2024).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>Occupancy 'yellow / red flag' (CREFC)</t>
+        </is>
+      </c>
+      <c r="B30" s="55" t="inlineStr">
+        <is>
+          <t>&lt;85% / &lt;75%</t>
+        </is>
+      </c>
+      <c r="C30" s="59" t="inlineStr">
+        <is>
+          <t>Credit-stress thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>Power utilization 'yellow / red flag' (CREFC)</t>
+        </is>
+      </c>
+      <c r="B31" s="55" t="inlineStr">
+        <is>
+          <t>&lt;60% / &lt;50%</t>
+        </is>
+      </c>
+      <c r="C31" s="59" t="inlineStr">
+        <is>
+          <t>Increasingly the key tracked metric.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="60" t="inlineStr">
+        <is>
+          <t>B.  NEOCLOUD (GPU compute-as-a-service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>GPU rental rates ($/GPU-hour, on-demand unless noted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>GPU SKU</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>CoreWeave (8x)</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Lambda</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Hyperscaler on-dmd</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Specialty rsv 3yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>A100 80GB</t>
+        </is>
+      </c>
+      <c r="B36" s="61" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C36" s="61" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="D36" s="44" t="inlineStr">
+        <is>
+          <t>$1.50 - $3.00</t>
+        </is>
+      </c>
+      <c r="E36" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>H100 SXM</t>
+        </is>
+      </c>
+      <c r="B37" s="61" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="C37" s="61" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="D37" s="44" t="inlineStr">
+        <is>
+          <t>$3.50 - $5.00</t>
+        </is>
+      </c>
+      <c r="E37" s="44" t="inlineStr">
+        <is>
+          <t>$1.70 - $2.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>H200 SXM</t>
+        </is>
+      </c>
+      <c r="B38" s="61" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="C38" s="61" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D38" s="44" t="inlineStr">
+        <is>
+          <t>$4.50 - $7.00</t>
+        </is>
+      </c>
+      <c r="E38" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>B200</t>
+        </is>
+      </c>
+      <c r="B39" s="61" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="C39" s="61" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="D39" s="44" t="inlineStr">
+        <is>
+          <t>$5.50+</t>
+        </is>
+      </c>
+      <c r="E39" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>GB200 NVL72</t>
+        </is>
+      </c>
+      <c r="B40" s="61" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C40" s="44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E40" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>GH200</t>
+        </is>
+      </c>
+      <c r="B41" s="61" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C41" s="61" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="D41" s="44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E41" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Discounts: reserved 1yr ~25-40% off on-demand; 3yr up to ~50%; spot ~50-80% below on-demand. CoreWeave bills 8-GPU clusters (premium for guaranteed capacity/orchestration); long-tail H100 ~$1.99-2.50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Utilization &amp; unit economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="D45" s="57" t="n"/>
+      <c r="E45" s="57" t="n"/>
+      <c r="F45" s="58" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="inlineStr">
+        <is>
+          <t>Debt-financed cluster break-even utilization</t>
+        </is>
+      </c>
+      <c r="B46" s="55" t="inlineStr">
+        <is>
+          <t>~65-70%</t>
+        </is>
+      </c>
+      <c r="C46" s="59" t="inlineStr">
+        <is>
+          <t>Little margin of safety (American Compute).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>1,024x H100 cluster @ 55% vs 85% util</t>
+        </is>
+      </c>
+      <c r="B47" s="55" t="inlineStr">
+        <is>
+          <t>-$330k vs +$340k /mo</t>
+        </is>
+      </c>
+      <c r="C47" s="59" t="inlineStr">
+        <is>
+          <t>Illustrates utilization sensitivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr">
+        <is>
+          <t>CoreWeave Model FLOPs Utilization (MFU)</t>
+        </is>
+      </c>
+      <c r="B48" s="55" t="inlineStr">
+        <is>
+          <t>50%+</t>
+        </is>
+      </c>
+      <c r="C48" s="59" t="inlineStr">
+        <is>
+          <t>Claimed vs industry typical 30-45%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>CoreWeave active power (Q1-2026)</t>
+        </is>
+      </c>
+      <c r="B49" s="55" t="inlineStr">
+        <is>
+          <t>&gt;1.0 GW</t>
+        </is>
+      </c>
+      <c r="C49" s="59" t="inlineStr">
+        <is>
+          <t>Plan: ~1.7 GW active in 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>CoreWeave contracted power (Q1-2026)</t>
+        </is>
+      </c>
+      <c r="B50" s="55" t="inlineStr">
+        <is>
+          <t>&gt;3.5 GW</t>
+        </is>
+      </c>
+      <c r="C50" s="59" t="inlineStr">
+        <is>
+          <t>Active/contracted ≈ 29% (energization gap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>CoreWeave revenue backlog (Mar-2026)</t>
+        </is>
+      </c>
+      <c r="B51" s="55" t="inlineStr">
+        <is>
+          <t>$99.4B</t>
+        </is>
+      </c>
+      <c r="C51" s="59" t="inlineStr">
+        <is>
+          <t>&gt;50% est. from Meta / OpenAI / hyperscalers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr">
+        <is>
+          <t>Bare-metal gross margin (pre-depreciation)</t>
+        </is>
+      </c>
+      <c r="B52" s="55" t="inlineStr">
+        <is>
+          <t>55-65%</t>
+        </is>
+      </c>
+      <c r="C52" s="59" t="inlineStr">
+        <is>
+          <t>Before heavy GPU depreciation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="inlineStr">
+        <is>
+          <t>Neocloud market size (2025)</t>
+        </is>
+      </c>
+      <c r="B53" s="55" t="inlineStr">
+        <is>
+          <t>$25B+</t>
+        </is>
+      </c>
+      <c r="C53" s="59" t="inlineStr">
+        <is>
+          <t>Q4-2025 $9B, +223% YoY (Synergy Research).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="inlineStr">
+        <is>
+          <t>Reserved-contract discounts</t>
+        </is>
+      </c>
+      <c r="B54" s="55" t="inlineStr">
+        <is>
+          <t>1yr 25-40%; 3yr up to ~50%</t>
+        </is>
+      </c>
+      <c r="C54" s="59" t="inlineStr">
+        <is>
+          <t>Spot 50-80% below on-demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Note: Meta's own contracted colocation rents and neocloud rates are confidential; figures above are market benchmarks used to frame Meta's economics. Owned/self-build effective cost is often quoted at ~$1.40-1.80/GPU-hr for a single GPU at ~70% utilization (before cluster/networking overhead).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="40">
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="D9"/>
+    <mergeCell ref="D8"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="D7"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="C27:F27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3633,269 +5265,269 @@
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="47" t="inlineStr">
+      <c r="A7" s="51" t="inlineStr">
         <is>
           <t>Prometheus</t>
         </is>
       </c>
-      <c r="B7" s="47" t="inlineStr">
+      <c r="B7" s="51" t="inlineStr">
         <is>
           <t>New Albany, Ohio</t>
         </is>
       </c>
-      <c r="C7" s="48" t="n">
+      <c r="C7" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="47" t="inlineStr">
+      <c r="D7" s="51" t="inlineStr">
         <is>
           <t>~1 GW by 2026</t>
         </is>
       </c>
-      <c r="E7" s="49" t="inlineStr">
+      <c r="E7" s="62" t="inlineStr">
         <is>
           <t>Owned self-build + leased + on-site gas</t>
         </is>
       </c>
-      <c r="F7" s="47" t="inlineStr">
+      <c r="F7" s="51" t="inlineStr">
         <is>
           <t>World's first ~1GW-scale AI training cluster; Meta pre-leased more capacity in H2-2024 than any hyperscaler, mostly Ohio; two 200MW behind-the-meter gas plants w/ Williams.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="47" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>Hyperion</t>
         </is>
       </c>
-      <c r="B8" s="47" t="inlineStr">
+      <c r="B8" s="51" t="inlineStr">
         <is>
           <t>Richland Parish, Louisiana</t>
         </is>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="47" t="inlineStr">
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>2 GW by 2030 (1.5 GW IT by 2027); scalable to 5 GW</t>
         </is>
       </c>
-      <c r="E8" s="50" t="inlineStr">
+      <c r="E8" s="63" t="inlineStr">
         <is>
           <t>JV-owned (Blue Owl 80% / Meta 20%), leased back to Meta</t>
         </is>
       </c>
-      <c r="F8" s="47" t="inlineStr">
+      <c r="F8" s="51" t="inlineStr">
         <is>
           <t>$27-30B Blue Owl JV finances the campus; fully leased by Meta. &gt;$10B Meta investment; ~4M+ sqft.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="47" t="inlineStr">
+      <c r="A9" s="51" t="inlineStr">
         <is>
           <t>Lebanon (El Paso project)</t>
         </is>
       </c>
-      <c r="B9" s="47" t="inlineStr">
+      <c r="B9" s="51" t="inlineStr">
         <is>
           <t>Lebanon, Indiana</t>
         </is>
       </c>
-      <c r="C9" s="48" t="n">
+      <c r="C9" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="47" t="inlineStr">
+      <c r="D9" s="51" t="inlineStr">
         <is>
           <t>~1 GW, from 2027</t>
         </is>
       </c>
-      <c r="E9" s="49" t="inlineStr">
+      <c r="E9" s="62" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
       </c>
-      <c r="F9" s="47" t="inlineStr">
+      <c r="F9" s="51" t="inlineStr">
         <is>
           <t>~4M sqft, 13 buildings, $10B+.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="47" t="inlineStr">
+      <c r="A10" s="51" t="inlineStr">
         <is>
           <t>Aiken (New Albany SC)</t>
         </is>
       </c>
-      <c r="B10" s="47" t="inlineStr">
+      <c r="B10" s="51" t="inlineStr">
         <is>
           <t>Aiken, South Carolina</t>
         </is>
       </c>
-      <c r="C10" s="51" t="inlineStr">
+      <c r="C10" s="52" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="D10" s="47" t="inlineStr">
+      <c r="D10" s="51" t="inlineStr">
         <is>
           <t>Under construction</t>
         </is>
       </c>
-      <c r="E10" s="49" t="inlineStr">
+      <c r="E10" s="62" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
       </c>
-      <c r="F10" s="47" t="inlineStr">
+      <c r="F10" s="51" t="inlineStr">
         <is>
           <t>AI-optimized campus, $800M+.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="47" t="inlineStr">
+      <c r="A11" s="51" t="inlineStr">
         <is>
           <t>El Paso</t>
         </is>
       </c>
-      <c r="B11" s="47" t="inlineStr">
+      <c r="B11" s="51" t="inlineStr">
         <is>
           <t>El Paso, Texas</t>
         </is>
       </c>
-      <c r="C11" s="51" t="inlineStr">
+      <c r="C11" s="52" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="D11" s="51" t="inlineStr">
         <is>
           <t>Under construction</t>
         </is>
       </c>
-      <c r="E11" s="49" t="inlineStr">
+      <c r="E11" s="62" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
       </c>
-      <c r="F11" s="47" t="inlineStr">
+      <c r="F11" s="51" t="inlineStr">
         <is>
           <t>AI-optimized; reporting ~$10B.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="47" t="inlineStr">
+      <c r="A12" s="51" t="inlineStr">
         <is>
           <t>Beaver Dam</t>
         </is>
       </c>
-      <c r="B12" s="47" t="inlineStr">
+      <c r="B12" s="51" t="inlineStr">
         <is>
           <t>Beaver Dam, Wisconsin</t>
         </is>
       </c>
-      <c r="C12" s="51" t="inlineStr">
+      <c r="C12" s="52" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="D12" s="47" t="inlineStr">
+      <c r="D12" s="51" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="E12" s="49" t="inlineStr">
+      <c r="E12" s="62" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
       </c>
-      <c r="F12" s="47" t="inlineStr">
+      <c r="F12" s="51" t="inlineStr">
         <is>
           <t>700k+ sqft, $1B+, closed-loop liquid cooling.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="47" t="inlineStr">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t>Cheyenne</t>
         </is>
       </c>
-      <c r="B13" s="47" t="inlineStr">
+      <c r="B13" s="51" t="inlineStr">
         <is>
           <t>Cheyenne, Wyoming</t>
         </is>
       </c>
-      <c r="C13" s="51" t="inlineStr">
+      <c r="C13" s="52" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="D13" s="47" t="inlineStr">
+      <c r="D13" s="51" t="inlineStr">
         <is>
           <t>Announced/UC</t>
         </is>
       </c>
-      <c r="E13" s="49" t="inlineStr">
+      <c r="E13" s="62" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
       </c>
-      <c r="F13" s="47" t="inlineStr">
+      <c r="F13" s="51" t="inlineStr">
         <is>
           <t>715k sqft.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="47" t="inlineStr">
+      <c r="A14" s="51" t="inlineStr">
         <is>
           <t>Tulsa</t>
         </is>
       </c>
-      <c r="B14" s="47" t="inlineStr">
+      <c r="B14" s="51" t="inlineStr">
         <is>
           <t>Tulsa, Oklahoma</t>
         </is>
       </c>
-      <c r="C14" s="51" t="inlineStr">
+      <c r="C14" s="52" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="D14" s="47" t="inlineStr">
+      <c r="D14" s="51" t="inlineStr">
         <is>
           <t>Announced Apr 2026</t>
         </is>
       </c>
-      <c r="E14" s="49" t="inlineStr">
+      <c r="E14" s="62" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
       </c>
-      <c r="F14" s="47" t="inlineStr">
+      <c r="F14" s="51" t="inlineStr">
         <is>
           <t>Meta's 32nd data center globally.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="52" t="inlineStr">
+      <c r="A15" s="64" t="inlineStr">
         <is>
           <t>Sum of quantified GW targets</t>
         </is>
       </c>
-      <c r="B15" s="53" t="n"/>
-      <c r="C15" s="54">
+      <c r="B15" s="65" t="n"/>
+      <c r="C15" s="66">
         <f>SUMIF(C7:C14,"&lt;&gt;n/d")</f>
         <v/>
       </c>
-      <c r="D15" s="53" t="n"/>
-      <c r="E15" s="53" t="n"/>
-      <c r="F15" s="53" t="n"/>
+      <c r="D15" s="65" t="n"/>
+      <c r="E15" s="65" t="n"/>
+      <c r="F15" s="65" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -3915,13 +5547,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3954,188 +5586,336 @@
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>• Capacity proxy: Data-center capacity is measured in electric power. Because Meta does not disclose a single owned-vs-leased MW figure, the owned/leased split uses ACTUAL electricity consumption (MWh/yr) as the realized-capacity proxy — the one metric Meta reports separately for owned sites and for leased facilities.</t>
+          <t>• Three procurement modes are tracked separately: (1) OWNED self-build; (2) LEASED COLOCATION — Meta leases space/power and owns the compute; (3) NEOCLOUD/CLOUD — Meta rents compute-as-a-service and the provider owns the GPUs. Owned + colocation are comparable in electricity (MWh); neocloud is a distinct $-denominated channel and is NOT additive with the electricity split.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>• Owned online data centers are reported individually by Meta (18 sites with material 2024 consumption). 'Leased data center facilities' and 'Other DC-related facilities' are each reported as single lines.</t>
+          <t>• Capacity proxy: Data-center capacity is measured in electric power. Because Meta does not disclose a single owned-vs-leased MW figure, the owned vs colocation split uses ACTUAL electricity consumption (MWh/yr) as the realized-capacity proxy — the one metric Meta reports separately for owned sites and for leased facilities.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>• Nameplate MW (Campus Detail) are third-party estimates (usdatamap) available only for a subset of sites; they understate installed power and exclude the AI expansion. Use directionally.</t>
+          <t>• Utilization &amp; rental rates (tab 6) are external market benchmarks (CBRE/JLL/CREFC for colocation; neocloud disclosures &amp; third-party price trackers for GPU rates). They frame Meta's economics but are NOT Meta's confidential contract terms.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>• AI build-out GW are announced targets / analyst estimates with multi-year phasing — NOT installed capacity.</t>
+          <t>• Owned online data centers are reported individually by Meta (18 sites with material 2024 consumption). 'Leased data center facilities' and 'Other DC-related facilities' are each reported as single lines.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>• Nameplate MW (Campus Detail) are third-party estimates (usdatamap) available only for a subset of sites; they understate installed power and exclude the AI expansion. Use directionally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>• AI build-out GW are announced targets / analyst estimates with multi-year phasing — NOT installed capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
           <t>• Owned campus counts vary by source and date (Meta cites '27-28 owned locations in operation or under construction'; Dgtl Infra lists 24 established campuses; newer sites e.g. Tulsa push counts higher). Reconciliation notes included where relevant.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>URL / detail</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="55" t="inlineStr">
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="67" t="inlineStr">
         <is>
           <t>Meta 2025 Environmental Data Index (FY2024)</t>
         </is>
       </c>
-      <c r="B13" s="47" t="inlineStr">
+      <c r="B15" s="51" t="inlineStr">
         <is>
           <t>https://sustainability.atmeta.com/wp-content/uploads/2025/10/Meta_2025-Environmental-Data-Index.pdf — per-site electricity (MWh), water, GHG; owned vs leased lines.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="55" t="inlineStr">
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="67" t="inlineStr">
         <is>
           <t>Meta 2025 Sustainability Report</t>
         </is>
       </c>
-      <c r="B14" s="47" t="inlineStr">
+      <c r="B16" s="51" t="inlineStr">
         <is>
           <t>https://www.smartenergydecisions.com/wp-content/uploads/2025/10/Meta_2025-Sustainability-Report_-compressed.pdf — '27 owned DC locations in operation or under construction'; new DC design uses less sqft per unit compute.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="55" t="inlineStr">
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="67" t="inlineStr">
         <is>
           <t>Meta — U.S. Data Centers list (2026)</t>
         </is>
       </c>
-      <c r="B15" s="47" t="inlineStr">
+      <c r="B17" s="51" t="inlineStr">
         <is>
           <t>https://datacenters.atmeta.com/wp-content/uploads/2026/04/V_Meta-United-States-Data-Centers.pdf — 28 U.S. data centers; Richland Parish &gt;2 GW.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="55" t="inlineStr">
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="67" t="inlineStr">
         <is>
           <t>Dgtl Infra — Meta data center locations</t>
         </is>
       </c>
-      <c r="B16" s="47" t="inlineStr">
+      <c r="B18" s="51" t="inlineStr">
         <is>
           <t>https://dgtlinfra.com/meta-data-center-locations-facebook/ — 24 campuses, 104 buildings, 53.4M sqft, ~$29.8B; leased markets; Digital Realty relationship.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="55" t="inlineStr">
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="67" t="inlineStr">
         <is>
           <t>SemiAnalysis — Meta Superintelligence (Jul 2025)</t>
         </is>
       </c>
-      <c r="B17" s="47" t="inlineStr">
+      <c r="B19" s="51" t="inlineStr">
         <is>
           <t>https://newsletter.semianalysis.com/p/meta-superintelligence-leadership-compute-talent-and-data — Prometheus 1GW, Hyperion, pre-leasing, on-site gas.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="55" t="inlineStr">
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="67" t="inlineStr">
         <is>
           <t>Data Center Frontier — Hyperion &amp; Prometheus</t>
         </is>
       </c>
-      <c r="B18" s="47" t="inlineStr">
+      <c r="B20" s="51" t="inlineStr">
         <is>
           <t>https://www.datacenterfrontier.com/hyperscale/article/55310441 — ownership/lease structure; 2 GW-&gt;5 GW; CAPEX.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="55" t="inlineStr">
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="67" t="inlineStr">
         <is>
           <t>AI Data Center Index — Meta operator report</t>
         </is>
       </c>
-      <c r="B19" s="47" t="inlineStr">
+      <c r="B21" s="51" t="inlineStr">
         <is>
           <t>https://aidatacenterindex.com/reports/operator/meta/ — ~15.8 GW tracked, 20 sites, ~50% operational, 5 countries.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="55" t="inlineStr">
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="67" t="inlineStr">
         <is>
           <t>usdatamap — Meta</t>
         </is>
       </c>
-      <c r="B20" s="47" t="inlineStr">
+      <c r="B22" s="51" t="inlineStr">
         <is>
           <t>https://usdatamap.com/company/meta — third-party per-site nameplate MW estimates (incomplete).</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="55" t="inlineStr">
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="67" t="inlineStr">
         <is>
           <t>CBRE North America DC Trends H2 2025</t>
         </is>
       </c>
-      <c r="B21" s="47" t="inlineStr">
+      <c r="B23" s="51" t="inlineStr">
         <is>
           <t>https://www.cbre.com/insights/books/north-america-data-center-trends-h2-2025 — Blue Owl JV; $27B Hyperion; market context.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="55" t="inlineStr">
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="67" t="inlineStr">
         <is>
           <t>Redact.dev — Facebook data center list (May 2026)</t>
         </is>
       </c>
-      <c r="B22" s="47" t="inlineStr">
+      <c r="B24" s="51" t="inlineStr">
         <is>
           <t>https://redact.dev/blog/full-list-of-known-and-upcoming-facebook-datacenters-as-of-may-2026 — campus sqft/investment; Lebanon ~1GW; Hyperion up to 5GW.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="67" t="inlineStr">
+        <is>
+          <t>CoreWeave — Meta $21B expansion (Apr 2026)</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>https://coreweave.com/news/coreweave-and-meta-announce-21-billion-expanded-ai-infrastructure-agreement — through Dec 2032; Vera Rubin; brings total to ~$35B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>Reuters — CoreWeave $14B Meta deal (Sep 2025)</t>
+        </is>
+      </c>
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/coreweave-signs-14-billion-ai-deal-with-meta-bloomberg-news-reports-2025-09-30/ — $14.2B through Dec 14 2031; GB300.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="67" t="inlineStr">
+        <is>
+          <t>CNBC — Meta +$21B CoreWeave (Apr 2026)</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2026/04/09/meta-commits-to-spending-additional-21-billion-with-coreweave-.html — 2027-2032; portfolio approach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>CNBC / Reuters / Bloomberg — Meta-Google Cloud (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="B28" s="51" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2025/08/21/google-scores-six-year-meta-cloud-deal-worth-over-10-billion.html — $10B+ over 6 yrs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="67" t="inlineStr">
+        <is>
+          <t>Alatirok — Neocloud Economics 2026</t>
+        </is>
+      </c>
+      <c r="B29" s="51" t="inlineStr">
+        <is>
+          <t>https://alatirok.com/neocloud-economics-2026/ — Nebius-Meta up to $27B ($12B + $15B option); CoreWeave $99.4B backlog / 3.5 GW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="67" t="inlineStr">
+        <is>
+          <t>CoreWeave Q1 FY2026 results</t>
+        </is>
+      </c>
+      <c r="B30" s="51" t="inlineStr">
+        <is>
+          <t>https://www.businesswire.com/news/home/20260507558197 — &gt;1 GW active, &gt;3.5 GW contracted power; Meta $21B; MFU context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>CBRE — N. America DC Trends H2 2025 &amp; Global 2026</t>
+        </is>
+      </c>
+      <c r="B31" s="51" t="inlineStr">
+        <is>
+          <t>https://www.cbre.com/insights/books/north-america-data-center-trends-h2-2025 — $196/kW/mo, 1.4% vacancy, metro rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>JLL — N. America DC Report YE 2025</t>
+        </is>
+      </c>
+      <c r="B32" s="51" t="inlineStr">
+        <is>
+          <t>https://www.jll.com/en-us/insights/market-dynamics/north-america-data-centers — 1% vacancy, 92% precommitted, 35+ GW UC, ~60% leased.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>CREFC — Data Center e-primer (2026)</t>
+        </is>
+      </c>
+      <c r="B33" s="51" t="inlineStr">
+        <is>
+          <t>https://www.crefc.org/common/Uploaded%20files/Learn/DataCenters-eprimer-2026.02.25.pdf — rate tiers by deal type; occupancy/power-utilization flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="67" t="inlineStr">
+        <is>
+          <t>Mercatus / DeployBase / Verda — GPU cloud pricing</t>
+        </is>
+      </c>
+      <c r="B34" s="51" t="inlineStr">
+        <is>
+          <t>https://www.mercatus-ai.com/blog/cloud-gpu-pricing — cross-provider $/GPU-hr by SKU (H100/H200/B200/GB200); reserved &amp; spot discounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>American Compute / ModulEdge — Neocloud unit economics</t>
+        </is>
+      </c>
+      <c r="B35" s="51" t="inlineStr">
+        <is>
+          <t>https://www.moduledge.com/blog/neocloud — ~70% break-even utilization; cluster P&amp;L sensitivity; margins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>Compiled: FY2024 basis. Prepared as an equity-research reference; verify against primary filings before use.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A9:B9"/>

</xml_diff>

<commit_message>
Add annualized CoreWeave & Nebius spend breakdown
- Split Nebius into Order #1 ($2.9B, Nov-2025) and the Mar-2026 Vera
  Rubin agreement ($12B firm + up to $15B contingent backstop) using
  SEC 6-K terms; CoreWeave initial ($14.2B, through Dec-2031) + expansion
  ($21B, 2027-2032).
- New Neocloud tab section: contract-level straight-line $/yr averages
  and an illustrative per-year run-rate matrix (2026-2032) with firm and
  incl.-backstop totals.
- Firm disclosed neocloud/cloud commitments now ~$60B (up to ~$75B);
  CoreWeave+Nebius run-rate ramps to ~$8-9B/yr firm (up to ~$12B) in
  2028-2031. Updated Cover and README.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/meta-compute-capacity/Meta_Compute_Capacity_Owned_vs_Leased.xlsx
+++ b/meta-compute-capacity/Meta_Compute_Capacity_Owned_vs_Leased.xlsx
@@ -82,7 +82,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +132,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF0FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -189,7 +194,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
       <top style="thin">
         <color rgb="00BFBFBF"/>
       </top>
@@ -200,9 +207,7 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
+      <right/>
       <top style="thin">
         <color rgb="00BFBFBF"/>
       </top>
@@ -215,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -314,7 +319,32 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -323,12 +353,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -601,7 +630,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2700000"/>
@@ -623,7 +652,7 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="2700000"/>
@@ -1004,7 +1033,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Headline #2 — neocloud / cloud commitments ($, off the electricity split)</t>
@@ -1012,7 +1041,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>CoreWeave ~$35B (initial $14.2B Sep-2025 + $21B expansion Apr-2026, through 2032; GB300 / Vera Rubin) | Nebius up to $27B ($12B fixed + $15B option) | Google Cloud $10B+ over 6 yrs (Aug-2025) | plus ongoing AWS &amp; Azure. ~$57B+ disclosed (up to ~$72B with options). These are compute rentals, NOT part of the owned-vs-colocation electricity split (different unit).</t>
+          <t>CoreWeave ~$35.2B (initial $14.2B Sep-2025 + $21B expansion Apr-2026, through 2032) | Nebius ~$14.9B firm ($2.9B Order #1 Nov-2025 + $12B Vera Rubin Mar-2026) plus up to $15B contingent backstop (=&gt; up to ~$27B) | Google Cloud $10B+ / 6 yrs | plus ongoing AWS &amp; Azure. ~$60B firm disclosed (up to ~$75B with the Nebius option). Straight-line, the CoreWeave + Nebius run-rate ramps to ~$8-9B/yr firm (up to ~$12B) in 2028-2031. These are compute rentals — NOT part of the owned-vs-colocation electricity split (different unit).</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1488,7 +1517,7 @@
     <row r="21">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Nebius — Order #1</t>
         </is>
       </c>
       <c r="B21" s="26" t="inlineStr">
@@ -1498,47 +1527,47 @@
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Nov 2025</t>
         </is>
       </c>
       <c r="D21" s="28" t="n">
-        <v>12</v>
+        <v>2.9</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>multi-year (+$15B option)</t>
+          <t>5 years (2026-2030)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>Google Cloud</t>
+          <t>Nebius — Vera Rubin agreement</t>
         </is>
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>Hyperscaler cloud</t>
+          <t>Neocloud (GPU-as-a-service)</t>
         </is>
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>Mar 2026</t>
         </is>
       </c>
       <c r="D22" s="28" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>6 years</t>
+          <t>5 years (from early 2027)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Amazon Web Services</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="B23" s="26" t="inlineStr">
@@ -1548,70 +1577,95 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="D23" s="27" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
+          <t>Aug 2025</t>
+        </is>
+      </c>
+      <c r="D23" s="28" t="n">
+        <v>10</v>
       </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>6 years</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="26" t="inlineStr">
         <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
           <t>Microsoft Azure</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>Hyperscaler cloud</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="D24" s="27" t="inlineStr">
+      <c r="D25" s="27" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="E24" s="26" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="29" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>Total disclosed neocloud/cloud commitments</t>
         </is>
       </c>
-      <c r="B25" s="30" t="n"/>
-      <c r="C25" s="30" t="n"/>
-      <c r="D25" s="31">
-        <f>SUMIF(D19:D24,"&lt;&gt;n/d")</f>
-        <v/>
-      </c>
-      <c r="E25" s="30" t="n"/>
-    </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="B26" s="30" t="n"/>
+      <c r="C26" s="30" t="n"/>
+      <c r="D26" s="31">
+        <f>SUMIF(D19:D25,"&lt;&gt;n/d")</f>
+        <v/>
+      </c>
+      <c r="E26" s="30" t="n"/>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Taxonomy: OWNED = Meta builds &amp; owns the DC and compute. COLOCATION = Meta leases space/power, owns the compute (in electricity split above, amber). NEOCLOUD/CLOUD = Meta rents GPU compute-as-a-service; the provider owns the GPUs &amp; building (this block, orange; measured in $, not MWh — not additive with the table above). See Neocloud &amp; Cloud and Utilization &amp; Rental Rates tabs.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Note: 'compute capacity' proxied by realized electricity consumption; see Cover &amp; Sources.</t>
         </is>
@@ -1619,7 +1673,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -3864,7 +3918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4019,7 +4073,7 @@
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="51" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Nebius — Order #1</t>
         </is>
       </c>
       <c r="B9" s="51" t="inlineStr">
@@ -4029,67 +4083,67 @@
       </c>
       <c r="C9" s="52" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Nov 2025</t>
         </is>
       </c>
       <c r="D9" s="53" t="n">
-        <v>12</v>
+        <v>2.9</v>
       </c>
       <c r="E9" s="51" t="inlineStr">
         <is>
-          <t>multi-year (+$15B option)</t>
+          <t>5 years (2026-2030)</t>
         </is>
       </c>
       <c r="F9" s="51" t="inlineStr">
         <is>
-          <t>Fixed dedicated compute</t>
+          <t>2 dedicated GPU clusters (deployed Dec-2025/Feb-2026)</t>
         </is>
       </c>
       <c r="G9" s="51" t="inlineStr">
         <is>
-          <t>Up to $27B including a $15B option exercisable at Nebius's discretion.</t>
+          <t>First Nebius-Meta order; SEC 6-K, Nov 1 2025.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="51" t="inlineStr">
         <is>
-          <t>Google Cloud</t>
+          <t>Nebius — Vera Rubin agreement</t>
         </is>
       </c>
       <c r="B10" s="51" t="inlineStr">
         <is>
-          <t>Hyperscaler cloud</t>
+          <t>Neocloud (GPU-as-a-service)</t>
         </is>
       </c>
       <c r="C10" s="52" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>Mar 2026</t>
         </is>
       </c>
       <c r="D10" s="53" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E10" s="51" t="inlineStr">
         <is>
-          <t>6 years</t>
+          <t>5 years (from early 2027)</t>
         </is>
       </c>
       <c r="F10" s="51" t="inlineStr">
         <is>
-          <t>Servers, storage, networking for AI</t>
+          <t>Dedicated NVIDIA Vera Rubin capacity</t>
         </is>
       </c>
       <c r="G10" s="51" t="inlineStr">
         <is>
-          <t>Minimum ~$10B; mainly AI infrastructure scaling.</t>
+          <t>Up to ~$27B: $12B firm dedicated + up to $15B contingent backstop for unsold capacity.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="51" t="inlineStr">
         <is>
-          <t>Amazon Web Services</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="B11" s="51" t="inlineStr">
@@ -4099,135 +4153,632 @@
       </c>
       <c r="C11" s="52" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="D11" s="52" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
+          <t>Aug 2025</t>
+        </is>
+      </c>
+      <c r="D11" s="53" t="n">
+        <v>10</v>
       </c>
       <c r="E11" s="51" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>6 years</t>
         </is>
       </c>
       <c r="F11" s="51" t="inlineStr">
         <is>
-          <t>Cloud infrastructure</t>
+          <t>Servers, storage, networking for AI</t>
         </is>
       </c>
       <c r="G11" s="51" t="inlineStr">
         <is>
-          <t>Long-standing; value undisclosed.</t>
+          <t>Minimum ~$10B; mainly AI infrastructure scaling.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="51" t="inlineStr">
         <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t>Hyperscaler cloud</t>
+        </is>
+      </c>
+      <c r="C12" s="52" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D12" s="52" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="F12" s="51" t="inlineStr">
+        <is>
+          <t>Cloud infrastructure</t>
+        </is>
+      </c>
+      <c r="G12" s="51" t="inlineStr">
+        <is>
+          <t>Long-standing; value undisclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="51" t="inlineStr">
+        <is>
           <t>Microsoft Azure</t>
         </is>
       </c>
-      <c r="B12" s="51" t="inlineStr">
+      <c r="B13" s="51" t="inlineStr">
         <is>
           <t>Hyperscaler cloud</t>
         </is>
       </c>
-      <c r="C12" s="52" t="inlineStr">
+      <c r="C13" s="52" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="D12" s="52" t="inlineStr">
+      <c r="D13" s="52" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="E12" s="51" t="inlineStr">
+      <c r="E13" s="51" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="F12" s="51" t="inlineStr">
+      <c r="F13" s="51" t="inlineStr">
         <is>
           <t>Cloud infrastructure</t>
         </is>
       </c>
-      <c r="G12" s="51" t="inlineStr">
+      <c r="G13" s="51" t="inlineStr">
         <is>
           <t>Long-standing; value undisclosed.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Total disclosed commitments</t>
         </is>
       </c>
-      <c r="B13" s="30" t="n"/>
-      <c r="C13" s="30" t="n"/>
-      <c r="D13" s="31">
-        <f>SUMIF(D7:D12,"&lt;&gt;n/d")</f>
-        <v/>
-      </c>
-      <c r="E13" s="30" t="n"/>
-      <c r="F13" s="30" t="n"/>
-      <c r="G13" s="30" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="B14" s="30" t="n"/>
+      <c r="C14" s="30" t="n"/>
+      <c r="D14" s="31">
+        <f>SUMIF(D7:D13,"&lt;&gt;n/d")</f>
+        <v/>
+      </c>
+      <c r="E14" s="30" t="n"/>
+      <c r="F14" s="30" t="n"/>
+      <c r="G14" s="30" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Context</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>• Meta describes this as a 'portfolio-based approach to infrastructure' — self-build + colocation + neocloud together.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>• CoreWeave total with Meta ~$35B (through 2032); CoreWeave overall backlog $99.4B (Mar-2026) on &gt;3.5 GW contracted power.</t>
+          <t>• Meta describes this as a 'portfolio-based approach to infrastructure' — self-build + colocation + neocloud together.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>• Nebius Meta deal up to $27B: $12B fixed dedicated compute + $15B option (exercisable by Nebius).</t>
+          <t>• CoreWeave total with Meta ~$35B (through 2032); CoreWeave overall backlog $99.4B (Mar-2026) on &gt;3.5 GW contracted power.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>• Google Cloud: $10B+ / 6 yrs; Meta historically also uses AWS and Azure (values undisclosed).</t>
+          <t>• Nebius Meta deal up to $27B: $12B fixed dedicated compute + $15B option (exercisable by Nebius).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>• Google Cloud: $10B+ / 6 yrs; Meta historically also uses AWS and Azure (values undisclosed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
           <t>• Neocloud GPU rental rates and utilization economics are on the 'Utilization &amp; Rental Rates' tab.</t>
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Estimated annualized spend — CoreWeave &amp; Nebius (straight-line = total ÷ term)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Total ($B)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Yrs</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Avg $B/yr</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>CoreWeave — initial</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>Sep 2025 - Dec 2031</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>~6</t>
+        </is>
+      </c>
+      <c r="E25" s="55" t="inlineStr">
+        <is>
+          <t>~2.3</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="G25" s="56" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>CoreWeave — expansion</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>21.0</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>2027 - 2032</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E26" s="55" t="inlineStr">
+        <is>
+          <t>~3.5</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="G26" s="56" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>Nebius — Order #1</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>2026 - 2030 (5-yr)</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E27" s="55" t="inlineStr">
+        <is>
+          <t>~0.6</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="G27" s="56" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>Nebius — dedicated (Vera Rubin)</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>2027 - 2031 (5-yr)</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E28" s="55" t="inlineStr">
+        <is>
+          <t>~2.4</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="G28" s="56" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="57" t="inlineStr">
+        <is>
+          <t>Nebius — unsold-capacity backstop</t>
+        </is>
+      </c>
+      <c r="B29" s="58" t="inlineStr">
+        <is>
+          <t>up to 15.0</t>
+        </is>
+      </c>
+      <c r="C29" s="58" t="inlineStr">
+        <is>
+          <t>~2027 - 2031 (5-yr)</t>
+        </is>
+      </c>
+      <c r="D29" s="58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E29" s="59" t="inlineStr">
+        <is>
+          <t>up to ~3.0</t>
+        </is>
+      </c>
+      <c r="F29" s="58" t="inlineStr">
+        <is>
+          <t>Contingent</t>
+        </is>
+      </c>
+      <c r="G29" s="60" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Illustrative per-year run-rate ($B, straight-line; actual spend is back-loaded as capacity deploys)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>2031</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>2032</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>CoreWeave — initial ($14.2B)</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="C33" s="28" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="D33" s="28" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="E33" s="28" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="F33" s="28" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H33" s="28" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="26" t="inlineStr">
+        <is>
+          <t>CoreWeave — expansion ($21B)</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="n"/>
+      <c r="C34" s="28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D34" s="28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E34" s="28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F34" s="28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H34" s="28" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>Nebius — Order #1 ($2.9B)</t>
+        </is>
+      </c>
+      <c r="B35" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C35" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="D35" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E35" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F35" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G35" s="28" t="n"/>
+      <c r="H35" s="28" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>Nebius — dedicated ($12B)</t>
+        </is>
+      </c>
+      <c r="B36" s="28" t="n"/>
+      <c r="C36" s="28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D36" s="28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E36" s="28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F36" s="28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H36" s="28" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="57" t="inlineStr">
+        <is>
+          <t>Nebius — backstop (up to $15B)</t>
+        </is>
+      </c>
+      <c r="B37" s="61" t="n"/>
+      <c r="C37" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F37" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="61" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>Firm total ($B/yr)</t>
+        </is>
+      </c>
+      <c r="B38" s="62">
+        <f>SUM(B33:B36)</f>
+        <v/>
+      </c>
+      <c r="C38" s="62">
+        <f>SUM(C33:C36)</f>
+        <v/>
+      </c>
+      <c r="D38" s="62">
+        <f>SUM(D33:D36)</f>
+        <v/>
+      </c>
+      <c r="E38" s="62">
+        <f>SUM(E33:E36)</f>
+        <v/>
+      </c>
+      <c r="F38" s="62">
+        <f>SUM(F33:F36)</f>
+        <v/>
+      </c>
+      <c r="G38" s="62">
+        <f>SUM(G33:G36)</f>
+        <v/>
+      </c>
+      <c r="H38" s="62">
+        <f>SUM(H33:H36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="63" t="inlineStr">
+        <is>
+          <t>Incl. Nebius backstop ($B/yr)</t>
+        </is>
+      </c>
+      <c r="B39" s="64">
+        <f>SUM(B33:B37)</f>
+        <v/>
+      </c>
+      <c r="C39" s="64">
+        <f>SUM(C33:C37)</f>
+        <v/>
+      </c>
+      <c r="D39" s="64">
+        <f>SUM(D33:D37)</f>
+        <v/>
+      </c>
+      <c r="E39" s="64">
+        <f>SUM(E33:E37)</f>
+        <v/>
+      </c>
+      <c r="F39" s="64">
+        <f>SUM(F33:F37)</f>
+        <v/>
+      </c>
+      <c r="G39" s="64">
+        <f>SUM(G33:G37)</f>
+        <v/>
+      </c>
+      <c r="H39" s="64">
+        <f>SUM(H33:H37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="56" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>How to read: figures are straight-line averages (contract total ÷ term). Actual cash spend/recognition is back-loaded — small in the first year of each contract and rising as GPU capacity is deployed and energized. Once fully ramped (~2028-2031), Meta's firm CoreWeave+Nebius run-rate is ~$8-9B/yr, or up to ~$12B/yr if Nebius's $15B unsold-capacity backstop is triggered. Excludes Google Cloud ($10B+/6yrs ≈ $1.7B/yr) and undisclosed AWS/Azure.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="16">
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A18:G18"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="F25:G25"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F26:G26"/>
     <mergeCell ref="A19:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4276,7 +4827,7 @@
       <c r="F2" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="54" t="inlineStr">
+      <c r="A4" s="65" t="inlineStr">
         <is>
           <t>A.  COLOCATION (space &amp; power leasing)</t>
         </is>
@@ -4327,12 +4878,12 @@
           <t>1-3 yr</t>
         </is>
       </c>
-      <c r="D7" s="55" t="inlineStr">
+      <c r="D7" s="66" t="inlineStr">
         <is>
           <t>$200 - $400</t>
         </is>
       </c>
-      <c r="E7" s="56" t="inlineStr">
+      <c r="E7" s="67" t="inlineStr">
         <is>
           <t>Highest unit price; smallest deployments.</t>
         </is>
@@ -4354,12 +4905,12 @@
           <t>5-10 yr</t>
         </is>
       </c>
-      <c r="D8" s="55" t="inlineStr">
+      <c r="D8" s="66" t="inlineStr">
         <is>
           <t>$150 - $250</t>
         </is>
       </c>
-      <c r="E8" s="56" t="inlineStr">
+      <c r="E8" s="67" t="inlineStr">
         <is>
           <t>Mid-size; typical enterprise / AI.</t>
         </is>
@@ -4381,12 +4932,12 @@
           <t>10-15 yr</t>
         </is>
       </c>
-      <c r="D9" s="55" t="inlineStr">
+      <c r="D9" s="66" t="inlineStr">
         <is>
           <t>$100 - $150</t>
         </is>
       </c>
-      <c r="E9" s="56" t="inlineStr">
+      <c r="E9" s="67" t="inlineStr">
         <is>
           <t>Largest deals, lowest unit rate — Meta's tier.</t>
         </is>
@@ -4420,8 +4971,8 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="E12" s="57" t="n"/>
-      <c r="F12" s="58" t="n"/>
+      <c r="E12" s="68" t="n"/>
+      <c r="F12" s="54" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
@@ -4439,7 +4990,7 @@
           <t>+6.6% YoY</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr">
+      <c r="D13" s="69" t="inlineStr">
         <is>
           <t>CBRE H2-2025 record; 4th straight annual rise.</t>
         </is>
@@ -4461,7 +5012,7 @@
           <t>+14.7% YoY</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr">
+      <c r="D14" s="69" t="inlineStr">
         <is>
           <t>Highest US primary rate (Q1-2026).</t>
         </is>
@@ -4483,7 +5034,7 @@
           <t>single-digit</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr">
+      <c r="D15" s="69" t="inlineStr">
         <is>
           <t>Largest US market.</t>
         </is>
@@ -4505,7 +5056,7 @@
           <t>+2% YoY</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr">
+      <c r="D16" s="69" t="inlineStr">
         <is>
           <t>Fast-growing; vacancy ~1%.</t>
         </is>
@@ -4527,7 +5078,7 @@
           <t>~flat</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr">
+      <c r="D17" s="69" t="inlineStr">
         <is>
           <t>Asking rents roughly unchanged YoY.</t>
         </is>
@@ -4549,7 +5100,7 @@
           <t>up YoY</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr">
+      <c r="D18" s="69" t="inlineStr">
         <is>
           <t>Highest European rate.</t>
         </is>
@@ -4571,7 +5122,7 @@
           <t>up YoY</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr">
+      <c r="D19" s="69" t="inlineStr">
         <is>
           <t>Highest APAC rate; supply-constrained.</t>
         </is>
@@ -4593,7 +5144,7 @@
           <t>up to +19% YoY</t>
         </is>
       </c>
-      <c r="D20" s="59" t="inlineStr">
+      <c r="D20" s="69" t="inlineStr">
         <is>
           <t>Large contiguous blocks command premiums.</t>
         </is>
@@ -4622,9 +5173,9 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="D23" s="57" t="n"/>
-      <c r="E23" s="57" t="n"/>
-      <c r="F23" s="58" t="n"/>
+      <c r="D23" s="68" t="n"/>
+      <c r="E23" s="68" t="n"/>
+      <c r="F23" s="54" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
@@ -4632,12 +5183,12 @@
           <t>Primary-market vacancy (CBRE, YE2025)</t>
         </is>
       </c>
-      <c r="B24" s="55" t="inlineStr">
+      <c r="B24" s="66" t="inlineStr">
         <is>
           <t>1.4%</t>
         </is>
       </c>
-      <c r="C24" s="59" t="inlineStr">
+      <c r="C24" s="69" t="inlineStr">
         <is>
           <t>Record low.</t>
         </is>
@@ -4649,12 +5200,12 @@
           <t>Primary-market vacancy (JLL, YE2025)</t>
         </is>
       </c>
-      <c r="B25" s="55" t="inlineStr">
+      <c r="B25" s="66" t="inlineStr">
         <is>
           <t>1.0%</t>
         </is>
       </c>
-      <c r="C25" s="59" t="inlineStr">
+      <c r="C25" s="69" t="inlineStr">
         <is>
           <t>2nd straight year; ~99% occupancy.</t>
         </is>
@@ -4666,12 +5217,12 @@
           <t>Under-construction precommitted (JLL)</t>
         </is>
       </c>
-      <c r="B26" s="55" t="inlineStr">
+      <c r="B26" s="66" t="inlineStr">
         <is>
           <t>92%</t>
         </is>
       </c>
-      <c r="C26" s="59" t="inlineStr">
+      <c r="C26" s="69" t="inlineStr">
         <is>
           <t>Binding leases or owner-occupied.</t>
         </is>
@@ -4683,12 +5234,12 @@
           <t>Under-construction that is leased (JLL)</t>
         </is>
       </c>
-      <c r="B27" s="55" t="inlineStr">
+      <c r="B27" s="66" t="inlineStr">
         <is>
           <t>~60%</t>
         </is>
       </c>
-      <c r="C27" s="59" t="inlineStr">
+      <c r="C27" s="69" t="inlineStr">
         <is>
           <t>Remaining ~40% owner-occupied.</t>
         </is>
@@ -4700,12 +5251,12 @@
           <t>N. America capacity under construction (JLL)</t>
         </is>
       </c>
-      <c r="B28" s="55" t="inlineStr">
+      <c r="B28" s="66" t="inlineStr">
         <is>
           <t>35+ GW</t>
         </is>
       </c>
-      <c r="C28" s="59" t="inlineStr">
+      <c r="C28" s="69" t="inlineStr">
         <is>
           <t>Extraordinary by historical standards.</t>
         </is>
@@ -4717,12 +5268,12 @@
           <t>Net absorption, primary markets 2025 (CBRE)</t>
         </is>
       </c>
-      <c r="B29" s="55" t="inlineStr">
+      <c r="B29" s="66" t="inlineStr">
         <is>
           <t>2,498 MW</t>
         </is>
       </c>
-      <c r="C29" s="59" t="inlineStr">
+      <c r="C29" s="69" t="inlineStr">
         <is>
           <t>Record; prior peak 1,810 MW (2024).</t>
         </is>
@@ -4734,12 +5285,12 @@
           <t>Occupancy 'yellow / red flag' (CREFC)</t>
         </is>
       </c>
-      <c r="B30" s="55" t="inlineStr">
+      <c r="B30" s="66" t="inlineStr">
         <is>
           <t>&lt;85% / &lt;75%</t>
         </is>
       </c>
-      <c r="C30" s="59" t="inlineStr">
+      <c r="C30" s="69" t="inlineStr">
         <is>
           <t>Credit-stress thresholds.</t>
         </is>
@@ -4751,19 +5302,19 @@
           <t>Power utilization 'yellow / red flag' (CREFC)</t>
         </is>
       </c>
-      <c r="B31" s="55" t="inlineStr">
+      <c r="B31" s="66" t="inlineStr">
         <is>
           <t>&lt;60% / &lt;50%</t>
         </is>
       </c>
-      <c r="C31" s="59" t="inlineStr">
+      <c r="C31" s="69" t="inlineStr">
         <is>
           <t>Increasingly the key tracked metric.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="60" t="inlineStr">
+      <c r="A33" s="70" t="inlineStr">
         <is>
           <t>B.  NEOCLOUD (GPU compute-as-a-service)</t>
         </is>
@@ -4809,10 +5360,10 @@
           <t>A100 80GB</t>
         </is>
       </c>
-      <c r="B36" s="61" t="n">
+      <c r="B36" s="71" t="n">
         <v>2.7</v>
       </c>
-      <c r="C36" s="61" t="n">
+      <c r="C36" s="71" t="n">
         <v>1.29</v>
       </c>
       <c r="D36" s="44" t="inlineStr">
@@ -4832,10 +5383,10 @@
           <t>H100 SXM</t>
         </is>
       </c>
-      <c r="B37" s="61" t="n">
+      <c r="B37" s="71" t="n">
         <v>6.16</v>
       </c>
-      <c r="C37" s="61" t="n">
+      <c r="C37" s="71" t="n">
         <v>3.29</v>
       </c>
       <c r="D37" s="44" t="inlineStr">
@@ -4855,10 +5406,10 @@
           <t>H200 SXM</t>
         </is>
       </c>
-      <c r="B38" s="61" t="n">
+      <c r="B38" s="71" t="n">
         <v>6.3</v>
       </c>
-      <c r="C38" s="61" t="n">
+      <c r="C38" s="71" t="n">
         <v>3.5</v>
       </c>
       <c r="D38" s="44" t="inlineStr">
@@ -4878,10 +5429,10 @@
           <t>B200</t>
         </is>
       </c>
-      <c r="B39" s="61" t="n">
+      <c r="B39" s="71" t="n">
         <v>8.6</v>
       </c>
-      <c r="C39" s="61" t="n">
+      <c r="C39" s="71" t="n">
         <v>4.99</v>
       </c>
       <c r="D39" s="44" t="inlineStr">
@@ -4901,7 +5452,7 @@
           <t>GB200 NVL72</t>
         </is>
       </c>
-      <c r="B40" s="61" t="n">
+      <c r="B40" s="71" t="n">
         <v>10.5</v>
       </c>
       <c r="C40" s="44" t="inlineStr">
@@ -4926,10 +5477,10 @@
           <t>GH200</t>
         </is>
       </c>
-      <c r="B41" s="61" t="n">
+      <c r="B41" s="71" t="n">
         <v>6.5</v>
       </c>
-      <c r="C41" s="61" t="n">
+      <c r="C41" s="71" t="n">
         <v>1.49</v>
       </c>
       <c r="D41" s="44" t="inlineStr">
@@ -4973,9 +5524,9 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="D45" s="57" t="n"/>
-      <c r="E45" s="57" t="n"/>
-      <c r="F45" s="58" t="n"/>
+      <c r="D45" s="68" t="n"/>
+      <c r="E45" s="68" t="n"/>
+      <c r="F45" s="54" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="24" t="inlineStr">
@@ -4983,12 +5534,12 @@
           <t>Debt-financed cluster break-even utilization</t>
         </is>
       </c>
-      <c r="B46" s="55" t="inlineStr">
+      <c r="B46" s="66" t="inlineStr">
         <is>
           <t>~65-70%</t>
         </is>
       </c>
-      <c r="C46" s="59" t="inlineStr">
+      <c r="C46" s="69" t="inlineStr">
         <is>
           <t>Little margin of safety (American Compute).</t>
         </is>
@@ -5000,12 +5551,12 @@
           <t>1,024x H100 cluster @ 55% vs 85% util</t>
         </is>
       </c>
-      <c r="B47" s="55" t="inlineStr">
+      <c r="B47" s="66" t="inlineStr">
         <is>
           <t>-$330k vs +$340k /mo</t>
         </is>
       </c>
-      <c r="C47" s="59" t="inlineStr">
+      <c r="C47" s="69" t="inlineStr">
         <is>
           <t>Illustrates utilization sensitivity.</t>
         </is>
@@ -5017,12 +5568,12 @@
           <t>CoreWeave Model FLOPs Utilization (MFU)</t>
         </is>
       </c>
-      <c r="B48" s="55" t="inlineStr">
+      <c r="B48" s="66" t="inlineStr">
         <is>
           <t>50%+</t>
         </is>
       </c>
-      <c r="C48" s="59" t="inlineStr">
+      <c r="C48" s="69" t="inlineStr">
         <is>
           <t>Claimed vs industry typical 30-45%.</t>
         </is>
@@ -5034,12 +5585,12 @@
           <t>CoreWeave active power (Q1-2026)</t>
         </is>
       </c>
-      <c r="B49" s="55" t="inlineStr">
+      <c r="B49" s="66" t="inlineStr">
         <is>
           <t>&gt;1.0 GW</t>
         </is>
       </c>
-      <c r="C49" s="59" t="inlineStr">
+      <c r="C49" s="69" t="inlineStr">
         <is>
           <t>Plan: ~1.7 GW active in 2026.</t>
         </is>
@@ -5051,12 +5602,12 @@
           <t>CoreWeave contracted power (Q1-2026)</t>
         </is>
       </c>
-      <c r="B50" s="55" t="inlineStr">
+      <c r="B50" s="66" t="inlineStr">
         <is>
           <t>&gt;3.5 GW</t>
         </is>
       </c>
-      <c r="C50" s="59" t="inlineStr">
+      <c r="C50" s="69" t="inlineStr">
         <is>
           <t>Active/contracted ≈ 29% (energization gap).</t>
         </is>
@@ -5068,12 +5619,12 @@
           <t>CoreWeave revenue backlog (Mar-2026)</t>
         </is>
       </c>
-      <c r="B51" s="55" t="inlineStr">
+      <c r="B51" s="66" t="inlineStr">
         <is>
           <t>$99.4B</t>
         </is>
       </c>
-      <c r="C51" s="59" t="inlineStr">
+      <c r="C51" s="69" t="inlineStr">
         <is>
           <t>&gt;50% est. from Meta / OpenAI / hyperscalers.</t>
         </is>
@@ -5085,12 +5636,12 @@
           <t>Bare-metal gross margin (pre-depreciation)</t>
         </is>
       </c>
-      <c r="B52" s="55" t="inlineStr">
+      <c r="B52" s="66" t="inlineStr">
         <is>
           <t>55-65%</t>
         </is>
       </c>
-      <c r="C52" s="59" t="inlineStr">
+      <c r="C52" s="69" t="inlineStr">
         <is>
           <t>Before heavy GPU depreciation.</t>
         </is>
@@ -5102,12 +5653,12 @@
           <t>Neocloud market size (2025)</t>
         </is>
       </c>
-      <c r="B53" s="55" t="inlineStr">
+      <c r="B53" s="66" t="inlineStr">
         <is>
           <t>$25B+</t>
         </is>
       </c>
-      <c r="C53" s="59" t="inlineStr">
+      <c r="C53" s="69" t="inlineStr">
         <is>
           <t>Q4-2025 $9B, +223% YoY (Synergy Research).</t>
         </is>
@@ -5119,12 +5670,12 @@
           <t>Reserved-contract discounts</t>
         </is>
       </c>
-      <c r="B54" s="55" t="inlineStr">
+      <c r="B54" s="66" t="inlineStr">
         <is>
           <t>1yr 25-40%; 3yr up to ~50%</t>
         </is>
       </c>
-      <c r="C54" s="59" t="inlineStr">
+      <c r="C54" s="69" t="inlineStr">
         <is>
           <t>Spot 50-80% below on-demand.</t>
         </is>
@@ -5283,7 +5834,7 @@
           <t>~1 GW by 2026</t>
         </is>
       </c>
-      <c r="E7" s="62" t="inlineStr">
+      <c r="E7" s="72" t="inlineStr">
         <is>
           <t>Owned self-build + leased + on-site gas</t>
         </is>
@@ -5313,7 +5864,7 @@
           <t>2 GW by 2030 (1.5 GW IT by 2027); scalable to 5 GW</t>
         </is>
       </c>
-      <c r="E8" s="63" t="inlineStr">
+      <c r="E8" s="73" t="inlineStr">
         <is>
           <t>JV-owned (Blue Owl 80% / Meta 20%), leased back to Meta</t>
         </is>
@@ -5343,7 +5894,7 @@
           <t>~1 GW, from 2027</t>
         </is>
       </c>
-      <c r="E9" s="62" t="inlineStr">
+      <c r="E9" s="72" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
@@ -5375,7 +5926,7 @@
           <t>Under construction</t>
         </is>
       </c>
-      <c r="E10" s="62" t="inlineStr">
+      <c r="E10" s="72" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
@@ -5407,7 +5958,7 @@
           <t>Under construction</t>
         </is>
       </c>
-      <c r="E11" s="62" t="inlineStr">
+      <c r="E11" s="72" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
@@ -5439,7 +5990,7 @@
           <t>2027</t>
         </is>
       </c>
-      <c r="E12" s="62" t="inlineStr">
+      <c r="E12" s="72" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
@@ -5471,7 +6022,7 @@
           <t>Announced/UC</t>
         </is>
       </c>
-      <c r="E13" s="62" t="inlineStr">
+      <c r="E13" s="72" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
@@ -5503,7 +6054,7 @@
           <t>Announced Apr 2026</t>
         </is>
       </c>
-      <c r="E14" s="62" t="inlineStr">
+      <c r="E14" s="72" t="inlineStr">
         <is>
           <t>Owned self-build</t>
         </is>
@@ -5515,19 +6066,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="64" t="inlineStr">
+      <c r="A15" s="74" t="inlineStr">
         <is>
           <t>Sum of quantified GW targets</t>
         </is>
       </c>
-      <c r="B15" s="65" t="n"/>
-      <c r="C15" s="66">
+      <c r="B15" s="75" t="n"/>
+      <c r="C15" s="76">
         <f>SUMIF(C7:C14,"&lt;&gt;n/d")</f>
         <v/>
       </c>
-      <c r="D15" s="65" t="n"/>
-      <c r="E15" s="65" t="n"/>
-      <c r="F15" s="65" t="n"/>
+      <c r="D15" s="75" t="n"/>
+      <c r="E15" s="75" t="n"/>
+      <c r="F15" s="75" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -5652,7 +6203,7 @@
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="67" t="inlineStr">
+      <c r="A15" s="77" t="inlineStr">
         <is>
           <t>Meta 2025 Environmental Data Index (FY2024)</t>
         </is>
@@ -5664,7 +6215,7 @@
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="67" t="inlineStr">
+      <c r="A16" s="77" t="inlineStr">
         <is>
           <t>Meta 2025 Sustainability Report</t>
         </is>
@@ -5676,7 +6227,7 @@
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="67" t="inlineStr">
+      <c r="A17" s="77" t="inlineStr">
         <is>
           <t>Meta — U.S. Data Centers list (2026)</t>
         </is>
@@ -5688,7 +6239,7 @@
       </c>
     </row>
     <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="67" t="inlineStr">
+      <c r="A18" s="77" t="inlineStr">
         <is>
           <t>Dgtl Infra — Meta data center locations</t>
         </is>
@@ -5700,7 +6251,7 @@
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="67" t="inlineStr">
+      <c r="A19" s="77" t="inlineStr">
         <is>
           <t>SemiAnalysis — Meta Superintelligence (Jul 2025)</t>
         </is>
@@ -5712,7 +6263,7 @@
       </c>
     </row>
     <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="67" t="inlineStr">
+      <c r="A20" s="77" t="inlineStr">
         <is>
           <t>Data Center Frontier — Hyperion &amp; Prometheus</t>
         </is>
@@ -5724,7 +6275,7 @@
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="67" t="inlineStr">
+      <c r="A21" s="77" t="inlineStr">
         <is>
           <t>AI Data Center Index — Meta operator report</t>
         </is>
@@ -5736,7 +6287,7 @@
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="67" t="inlineStr">
+      <c r="A22" s="77" t="inlineStr">
         <is>
           <t>usdatamap — Meta</t>
         </is>
@@ -5748,7 +6299,7 @@
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="67" t="inlineStr">
+      <c r="A23" s="77" t="inlineStr">
         <is>
           <t>CBRE North America DC Trends H2 2025</t>
         </is>
@@ -5760,7 +6311,7 @@
       </c>
     </row>
     <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="67" t="inlineStr">
+      <c r="A24" s="77" t="inlineStr">
         <is>
           <t>Redact.dev — Facebook data center list (May 2026)</t>
         </is>
@@ -5772,7 +6323,7 @@
       </c>
     </row>
     <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="67" t="inlineStr">
+      <c r="A25" s="77" t="inlineStr">
         <is>
           <t>CoreWeave — Meta $21B expansion (Apr 2026)</t>
         </is>
@@ -5784,7 +6335,7 @@
       </c>
     </row>
     <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="67" t="inlineStr">
+      <c r="A26" s="77" t="inlineStr">
         <is>
           <t>Reuters — CoreWeave $14B Meta deal (Sep 2025)</t>
         </is>
@@ -5796,7 +6347,7 @@
       </c>
     </row>
     <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="67" t="inlineStr">
+      <c r="A27" s="77" t="inlineStr">
         <is>
           <t>CNBC — Meta +$21B CoreWeave (Apr 2026)</t>
         </is>
@@ -5808,7 +6359,7 @@
       </c>
     </row>
     <row r="28" ht="40" customHeight="1">
-      <c r="A28" s="67" t="inlineStr">
+      <c r="A28" s="77" t="inlineStr">
         <is>
           <t>CNBC / Reuters / Bloomberg — Meta-Google Cloud (Aug 2025)</t>
         </is>
@@ -5820,7 +6371,7 @@
       </c>
     </row>
     <row r="29" ht="40" customHeight="1">
-      <c r="A29" s="67" t="inlineStr">
+      <c r="A29" s="77" t="inlineStr">
         <is>
           <t>Alatirok — Neocloud Economics 2026</t>
         </is>
@@ -5832,7 +6383,7 @@
       </c>
     </row>
     <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="67" t="inlineStr">
+      <c r="A30" s="77" t="inlineStr">
         <is>
           <t>CoreWeave Q1 FY2026 results</t>
         </is>
@@ -5844,7 +6395,7 @@
       </c>
     </row>
     <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="67" t="inlineStr">
+      <c r="A31" s="77" t="inlineStr">
         <is>
           <t>CBRE — N. America DC Trends H2 2025 &amp; Global 2026</t>
         </is>
@@ -5856,7 +6407,7 @@
       </c>
     </row>
     <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="67" t="inlineStr">
+      <c r="A32" s="77" t="inlineStr">
         <is>
           <t>JLL — N. America DC Report YE 2025</t>
         </is>
@@ -5868,7 +6419,7 @@
       </c>
     </row>
     <row r="33" ht="40" customHeight="1">
-      <c r="A33" s="67" t="inlineStr">
+      <c r="A33" s="77" t="inlineStr">
         <is>
           <t>CREFC — Data Center e-primer (2026)</t>
         </is>
@@ -5880,7 +6431,7 @@
       </c>
     </row>
     <row r="34" ht="40" customHeight="1">
-      <c r="A34" s="67" t="inlineStr">
+      <c r="A34" s="77" t="inlineStr">
         <is>
           <t>Mercatus / DeployBase / Verda — GPU cloud pricing</t>
         </is>
@@ -5892,7 +6443,7 @@
       </c>
     </row>
     <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="67" t="inlineStr">
+      <c r="A35" s="77" t="inlineStr">
         <is>
           <t>American Compute / ModulEdge — Neocloud unit economics</t>
         </is>

</xml_diff>